<commit_message>
feat: optimize dictionary for banking context examples
- Improved dictionary entries to better align with banking-related scenarios
- Enhanced example generation with more relevant placeholder values
- Increased accuracy and contextual fit for rule engine outputs
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="90">
   <si>
     <t>document</t>
   </si>
@@ -31,290 +31,343 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu theo primary key</t>
+    <t>customer_account | Tra cứu theo khóa chính</t>
   </si>
   <si>
     <t>customer_account | Tra cứu theo số định danh</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu theo mã số</t>
+    <t>customer_account | Tra cứu theo số</t>
   </si>
   <si>
     <t>customer_account | Lọc theo phân loại tài khoản</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu theo app/web</t>
+    <t>customer_account | Tìm kiếm theo đánh dấu tài khoản chính</t>
   </si>
   <si>
     <t>customer_account | Lọc theo ví dụ: a - active, i - inactive, c - closed</t>
   </si>
   <si>
-    <t>customer_account | Lọc theo trạng thái xác thực tài khoản</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo kết quả</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo thời gian (hôm)</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo mã chi nhánh nơi quản lý tài khoản này.</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo ví dụ: 411122****1234</t>
+    <t>customer_account | Lọc theo trạng thái</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>customer_account | Tìm kiếm theo độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo thời gian (thời gian)</t>
+  </si>
+  <si>
+    <t>customer_account | Tìm kiếm theo tên tài khoản</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo nơi mở</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu theo số thẻ được che bớt</t>
   </si>
   <si>
     <t>customer_account | Tra cứu theo customer number</t>
   </si>
   <si>
-    <t>customer_account | Lọc account_class theo Thời gian</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên primary key</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên số định danh</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên mã số</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách tài khoản theo nhóm phân loại tài khoản</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên app/web</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách tài khoản theo nhóm ví dụ: a - active, i - inactive, c - closed</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách tài khoản theo nhóm trạng thái xác thực tài khoản</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách tài khoản theo nhóm kết quả</t>
-  </si>
-  <si>
-    <t>Sao kê lịch sử tài khoản trong khoảng thời gian</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên mã chi nhánh nơi quản lý tài khoản này.</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên ví dụ: 411122****1234</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác tài khoản dựa trên customer number</t>
-  </si>
-  <si>
-    <t>Kết hợp lọc theo account_class và khoảng ngày tháng</t>
-  </si>
-  <si>
-    <t>Thông tin về tài khoản số 19423
-Xem chi tiết 65990
-Vui lòng Tra cứu thông tin chi tiết của tài khoản có primary key là 19498
-Check primary key 76880
-Tìm kiếm tài khoản ứng với số 28585
-Tra cứu tài khoản theo primary key 4779
-tài khoản 33674
-primary key 20351 là của ai?
-Hãy hiển thị dữ liệu bản ghi tài khoản với primary key 5597</t>
-  </si>
-  <si>
-    <t>Thông tin về tài khoản số 97497
-tài khoản 36624
-Hãy hiển thị dữ liệu bản ghi tài khoản với số định danh 61261
-Tra cứu tài khoản theo số định danh 18032
-Check số định danh 53205
-Tìm kiếm tài khoản ứng với số 64839
-số định danh 46358 là của ai?
-Vui lòng Tra cứu thông tin chi tiết của tài khoản có số định danh là 77531
-Xem chi tiết 30875</t>
-  </si>
-  <si>
-    <t>Xem chi tiết 3373226124203
-Hãy hiển thị dữ liệu bản ghi tài khoản với mã số 5584158087876
-Check mã số 1926512079783
-mã số 1839574558045 là của ai?
-Tra cứu tài khoản theo mã số 5430143585294
-tài khoản 3616554397837
-Thông tin về tài khoản số 9742091729715
-Tìm kiếm tài khoản ứng với số 5982441548805
-Vui lòng Tra cứu thông tin chi tiết của tài khoản có mã số là 5194884648074</t>
-  </si>
-  <si>
-    <t>Những tài khoản nào là đã?
-Lọc các tài khoản đang ở trạng thái để
-Hãy liệt kê danh sách các tài khoản có phân loại tài khoản là đang
-Danh sách chưa
-Cho xem danh sách tài khoản được
-Trích xuất báo cáo các tài khoản thuộc loại nhưng
-Tìm tất cả tài khoản loại cách</t>
-  </si>
-  <si>
-    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có app/web là 64882
-Hãy hiển thị dữ liệu bản ghi tài khoản với app/web 53430
-app/web 14635 là của ai?
-tài khoản 99948
-Tra cứu tài khoản theo app/web 41805
-Thông tin về tài khoản số 77216
-Check app/web 26738
-Xem chi tiết 40887
-Tìm kiếm tài khoản ứng với số 45946</t>
-  </si>
-  <si>
-    <t>Tìm tất cả tài khoản loại có
-Trích xuất báo cáo các tài khoản thuộc loại như
-Những tài khoản nào là người?
-Danh sách để
-Hãy liệt kê danh sách các tài khoản có ví dụ: a - active, i - inactive, c - closed là giữa
-Cho xem danh sách tài khoản từng
-Lọc các tài khoản đang ở trạng thái cho</t>
-  </si>
-  <si>
-    <t>Danh sách cũng
-Hãy liệt kê danh sách các tài khoản có trạng thái xác thực tài khoản là sẽ
-Cho xem danh sách tài khoản từ
-Những tài khoản nào là một?
-Trích xuất báo cáo các tài khoản thuộc loại không
-Tìm tất cả tài khoản loại theo
-Lọc các tài khoản đang ở trạng thái như</t>
-  </si>
-  <si>
-    <t>Tìm tất cả tài khoản loại vậy
-Lọc các tài khoản đang ở trạng thái với
-Trích xuất báo cáo các tài khoản thuộc loại đang
-Danh sách đến
-Hãy liệt kê danh sách các tài khoản có kết quả là có
-Cho xem danh sách tài khoản từng
-Những tài khoản nào là như?</t>
-  </si>
-  <si>
-    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có số định danh là 5960
-Tra cứu tài khoản theo số định danh 5078
-Check số định danh 74850
-số định danh 76495 là của ai?
-tài khoản 28897
-Xem chi tiết 59138
-Tìm kiếm tài khoản ứng với số 79318
-Thông tin về tài khoản số 1471
-Hãy hiển thị dữ liệu bản ghi tài khoản với số định danh 33246</t>
-  </si>
-  <si>
-    <t>Xem biến động tài khoản giữa 2025-12-28 và hôm nay
-Truy xuất lịch sử tài khoản trong khoảng thời gian từ 2025-08-29 đến hôm nay
-Lịch sử tài khoản 2025-03-13 đến hôm nay
-Sao kê tài khoản từ 2025-05-11 - hôm nay
-Những tài khoản nào diễn ra từ 2025-08-14 đến hôm nay?
-Liệt kê các giao dịch phát sinh từ ngày 2025-06-08 tới ngày hôm nay
-Kiểm tra tài khoản trong ngày 2025-02-05</t>
-  </si>
-  <si>
-    <t>tài khoản 5261871663267
-Tìm kiếm tài khoản ứng với số 9814480449297
-Hãy hiển thị dữ liệu bản ghi tài khoản với mã chi nhánh nơi quản lý tài khoản này. 1989982134478
-Thông tin về tài khoản số 8195806222815
-Tra cứu tài khoản theo mã chi nhánh nơi quản lý tài khoản này. 7213784096727
-Xem chi tiết 5281190454958
-Vui lòng Tra cứu thông tin chi tiết của tài khoản có mã chi nhánh nơi quản lý tài khoản này. là 7741924180987
-mã chi nhánh nơi quản lý tài khoản này. 1201783575956 là của ai?
-Check mã chi nhánh nơi quản lý tài khoản này. 5460797752316</t>
-  </si>
-  <si>
-    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có ví dụ: 411122****1234 là 5782560692367965
-Check ví dụ: 411122****1234 5423620394758073
-Xem chi tiết 4976505306348433
-Thông tin về tài khoản số 4513541511545584
-ví dụ: 411122****1234 4829723157040011 là của ai?
-tài khoản 5077291858859586
-Hãy hiển thị dữ liệu bản ghi tài khoản với ví dụ: 411122****1234 5455835439336649
-Tra cứu tài khoản theo ví dụ: 411122****1234 4863545002647533
-Tìm kiếm tài khoản ứng với số 5172369045882021</t>
-  </si>
-  <si>
-    <t>Vui lòng Tra cứu thông tin chi tiết của tài khoản có customer number là 40802
-tài khoản 82265
-customer number 80059 là của ai?
-Check customer number 47670
-Hãy hiển thị dữ liệu bản ghi tài khoản với customer number 97195
-Tìm kiếm tài khoản ứng với số 15671
-Xem chi tiết 74120
-Thông tin về tài khoản số 48129
-Tra cứu tài khoản theo customer number 71565</t>
-  </si>
-  <si>
-    <t>số định danh 79852 là của ai?
-Tìm kiếm tài khoản ứng với số 8054
-Hãy hiển thị dữ liệu bản ghi tài khoản với số định danh 62147
-Vui lòng Tra cứu thông tin chi tiết của tài khoản có số định danh là 51604
-Tra cứu tài khoản theo số định danh 73132
-tài khoản 87272
-Check số định danh 14324
-Thông tin về tài khoản số 58844
-Xem chi tiết 90378</t>
-  </si>
-  <si>
-    <t>Truy xuất lịch sử tài khoản trong khoảng thời gian từ 2026-01-07 đến hôm nay
-Kiểm tra tài khoản trong ngày 2025-07-06
-Xem biến động tài khoản giữa 2025-08-15 và hôm nay
-Sao kê tài khoản từ 2025-10-12 - hôm nay
-Lịch sử tài khoản 2025-03-25 đến hôm nay
-Liệt kê các giao dịch phát sinh từ ngày 2025-06-13 tới ngày hôm nay
-Những tài khoản nào diễn ra từ 2025-03-15 đến hôm nay?</t>
-  </si>
-  <si>
-    <t>Sao kê tài khoản loại trong từ ngày 2025-04-21 tới hôm nay
-Lọc các tài khoản điều diễn ra từ 2025-08-02 đến hôm nay
-Liệt kê tài khoản thay phát sinh ngày 2025-11-04
-Tìm tài khoản đúng hôm 2025-08-13
-Xem tài khoản có account_class là khi trong khoảng 2025-07-02 - hôm nay</t>
-  </si>
-  <si>
-    <t>id, primary key, tìm kiếm</t>
-  </si>
-  <si>
-    <t>core_customer_id, số định danh, tìm kiếm</t>
-  </si>
-  <si>
-    <t>account_no, mã số, tìm kiếm</t>
-  </si>
-  <si>
-    <t>account_class, phân loại tài khoản, danh sách</t>
-  </si>
-  <si>
-    <t>order_no, app/web, tìm kiếm</t>
-  </si>
-  <si>
-    <t>status, ví dụ: a - active, i - inactive, c - closed, danh sách</t>
-  </si>
-  <si>
-    <t>verify_status, trạng thái xác thực tài khoản, danh sách</t>
-  </si>
-  <si>
-    <t>check_status, kết quả, danh sách</t>
-  </si>
-  <si>
-    <t>channel_id, số định danh, tìm kiếm</t>
-  </si>
-  <si>
-    <t>create_date, thời gian, ngày tháng</t>
-  </si>
-  <si>
-    <t>account_branch, mã chi nhánh nơi quản lý tài khoản này., tìm kiếm</t>
-  </si>
-  <si>
-    <t>card_mask, ví dụ: 411122****1234, tìm kiếm</t>
-  </si>
-  <si>
-    <t>customer_no, customer number, tìm kiếm</t>
-  </si>
-  <si>
-    <t>system_id, số định danh, tìm kiếm</t>
-  </si>
-  <si>
-    <t>end_date, thời gian, ngày tháng</t>
-  </si>
-  <si>
-    <t>account_class, create_date, lọc đa điều kiện</t>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên khóa chính (id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (core_customer_id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số (account_no)</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách customer_account được phân nhóm bởi phân loại tài khoản. Ví dụ: phân loại tài khoản A, B...</t>
+  </si>
+  <si>
+    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong đánh dấu tài khoản chính</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số (order_no)</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách customer_account được phân nhóm bởi ví dụ: a - active, i - inactive, c - closed. Ví dụ: ví dụ: a - active, i - inactive, c - closed A, B...</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách customer_account được phân nhóm bởi trạng thái. Ví dụ: trạng thái A, B...</t>
+  </si>
+  <si>
+    <t>Liệt kê danh sách customer_account được phân nhóm bởi trạng thái kiểm tra. Ví dụ: trạng thái kiểm tra A, B...</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (channel_id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử customer_account trong một khoảng thời gian cụ thể (Từ ngày... đến ngày...)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong tên tài khoản</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên nơi mở (account_branch)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số thẻ được che bớt (card_mask)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên customer number (customer_no)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (system_id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm customer_account ứng với số 913895
+customer_account 560216
+Hãy hiển thị dữ liệu bản ghi customer_account với khóa chính 430935
+Check khóa chính 151612
+Thông tin về customer_account số 193999
+Vui lòng Tra cứu thông tin chi tiết của customer_account có khóa chính là 446305
+Tra cứu customer_account theo khóa chính 296445
+Xem chi tiết 825570
+khóa chính 922006 là của ai?</t>
+  </si>
+  <si>
+    <t>số định danh 127358 là của ai?
+Vui lòng Tra cứu thông tin chi tiết của customer_account có số định danh là 908149
+Thông tin về customer_account số 424316
+Tìm kiếm customer_account ứng với số 227326
+customer_account 704056
+Hãy hiển thị dữ liệu bản ghi customer_account với số định danh 881481
+Xem customer_account theo số định danh 824627
+Xem chi tiết 201516
+Check số định danh 118911</t>
+  </si>
+  <si>
+    <t>Thông tin về customer_account số 416933
+Xem chi tiết 413219
+Check số 655034
+customer_account 381069
+số 523447 là của ai?
+Tìm kiếm customer_account ứng với số 209514
+Hãy hiển thị dữ liệu bản ghi customer_account với số 537525
+Xem customer_account theo số 630521
+Vui lòng Tra cứu thông tin chi tiết của customer_account có số là 124949</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có phân loại tài khoản là hơn
+Tìm tất cả customer_account loại để
+Cho xem danh sách customer_account đã
+Những customer_account nào là cũng?
+Lọc các customer_account đang ở trạng thái đến
+Trích xuất báo cáo các customer_account thuộc loại chưa
+Danh sách vậy</t>
+  </si>
+  <si>
+    <t>Check đánh dấu tài khoản chính từ
+Hãy hiển thị dữ liệu bản ghi customer_account với đánh dấu tài khoản chính đã
+đánh dấu tài khoản chính điều là của ai?
+customer_account nhiều
+Tra cứu customer_account theo đánh dấu tài khoản chính cũng
+Tìm kiếm customer_account ứng với số tự
+Xem chi tiết từ
+Thông tin về customer_account số đã
+Vui lòng Xem thông tin chi tiết của customer_account có đánh dấu tài khoản chính là của</t>
+  </si>
+  <si>
+    <t>Tìm kiếm customer_account ứng với số 386870
+Check số 909408
+Xem customer_account theo số 951122
+Vui lòng Xem thông tin chi tiết của customer_account có số là 277145
+customer_account 329132
+số 534690 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với số 840060
+Xem chi tiết 544336
+Thông tin về customer_account số 440238</t>
+  </si>
+  <si>
+    <t>Những customer_account nào là CŨNG?
+Trích xuất báo cáo các customer_account thuộc loại SỐ
+Tìm tất cả customer_account loại ĐƯỢC
+Lọc các customer_account đang ở trạng thái LỚN
+Hãy liệt kê danh sách các customer_account có ví dụ: a - active, i - inactive, c - closed là CÓ
+customer_account thất bại
+danh sách customer_account thất bại
+Danh sách DƯỚI
+Cho xem danh sách customer_account ĐỂ</t>
+  </si>
+  <si>
+    <t>Tìm tất cả customer_account loại TRONG
+Những customer_account nào là LÀM?
+Cho xem danh sách customer_account NÀY
+danh sách customer_account bị treo
+customer_account bị treo
+Hãy liệt kê danh sách các customer_account có trạng thái là SẼ
+Trích xuất báo cáo các customer_account thuộc loại TẠI
+Lọc các customer_account đang ở trạng thái BÊN
+Danh sách TRONG</t>
+  </si>
+  <si>
+    <t>Những customer_account nào là CŨNG?
+Cho xem danh sách customer_account SAU
+Tìm tất cả customer_account loại CỦA
+customer_account đang chờ
+Lọc các customer_account đang ở trạng thái HƠN
+Hãy liệt kê danh sách các customer_account có trạng thái kiểm tra là THEO
+danh sách customer_account đang chờ
+Danh sách KHIẾN
+Trích xuất báo cáo các customer_account thuộc loại LÀ</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số định danh THẾ
+Thông tin về customer_account số HƠN
+Check số định danh KHÔNG
+Vui lòng Xem thông tin chi tiết của customer_account có số định danh là VỀ
+Tra cứu customer_account theo số định danh VÀI
+số định danh ĐẾN là của ai?
+Tìm kiếm customer_account ứng với số CÓ
+customer_account NHƯ
+Xem chi tiết THẾ</t>
+  </si>
+  <si>
+    <t>Xem customer_account theo độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. trong
+customer_account giống
+Hãy hiển thị dữ liệu bản ghi customer_account với độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. nhiều
+Tìm kiếm customer_account ứng với số vài
+Check độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. thay
+Vui lòng Tra cứu thông tin chi tiết của customer_account có độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. là hơn
+độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. khiến là của ai?
+Xem chi tiết người
+Thông tin về customer_account số là</t>
+  </si>
+  <si>
+    <t>Những customer_account nào diễn ra từ 2026-01-23 đến hôm nay?
+Xem biến động customer_account giữa 2026-01-14 và hôm nay
+Lịch sử customer_account 2026-01-17 đến hôm nay
+Sao kê customer_account từ 2026-01-16 - hôm nay
+Kiểm tra customer_account trong ngày 2026-01-15
+Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-10 đến hôm nay
+Liệt kê các giao dịch phát sinh từ ngày 2026-01-02 tới ngày hôm nay</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với tên tài khoản hơn
+Thông tin về customer_account số có
+Xem chi tiết các
+Tìm kiếm customer_account ứng với số cách
+Xem customer_account theo tên tài khoản lớn
+Vui lòng Tìm thông tin chi tiết của customer_account có tên tài khoản là đến
+Check tên tài khoản nhiều
+customer_account tự
+tên tài khoản hơn là của ai?</t>
+  </si>
+  <si>
+    <t>Vui lòng Tìm thông tin chi tiết của customer_account có nơi mở là vậy
+Check nơi mở lớn
+Xem chi tiết của
+Thông tin về customer_account số đang
+Hãy hiển thị dữ liệu bản ghi customer_account với nơi mở để
+nơi mở sẽ là của ai?
+customer_account bạn
+Tìm kiếm customer_account ứng với số lớn
+Xem customer_account theo nơi mở người</t>
+  </si>
+  <si>
+    <t>Check số thẻ được che bớt rất
+Hãy hiển thị dữ liệu bản ghi customer_account với số thẻ được che bớt các
+Tìm kiếm customer_account ứng với số từng
+Thông tin về customer_account số vì
+Tìm customer_account theo số thẻ được che bớt về
+customer_account giống
+Xem chi tiết tôi
+số thẻ được che bớt theo là của ai?
+Vui lòng Tìm thông tin chi tiết của customer_account có số thẻ được che bớt là cho</t>
+  </si>
+  <si>
+    <t>Tra cứu customer_account theo customer number 621908
+Tìm kiếm customer_account ứng với số 541697
+Thông tin về customer_account số 190775
+customer_account 484641
+Vui lòng Xem thông tin chi tiết của customer_account có customer number là 913734
+customer number 904988 là của ai?
+Xem chi tiết 998904
+Check customer number 354129
+Hãy hiển thị dữ liệu bản ghi customer_account với customer number 582931</t>
+  </si>
+  <si>
+    <t>Vui lòng Tra cứu thông tin chi tiết của customer_account có số định danh là 950436
+Tìm kiếm customer_account ứng với số 164102
+Thông tin về customer_account số 724600
+Check số định danh 410234
+Xem chi tiết 436611
+customer_account 824049
+số định danh 410017 là của ai?
+Tra cứu customer_account theo số định danh 389848
+Hãy hiển thị dữ liệu bản ghi customer_account với số định danh 118131</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account từ 2026-01-12 - hôm nay
+Kiểm tra customer_account trong ngày 2026-01-04
+Xem biến động customer_account giữa 2025-12-30 và hôm nay
+Những customer_account nào diễn ra từ 2026-01-03 đến hôm nay?
+Lịch sử customer_account 2026-01-09 đến hôm nay
+Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-13 đến hôm nay
+Liệt kê các giao dịch phát sinh từ ngày 2026-01-05 tới ngày hôm nay</t>
+  </si>
+  <si>
+    <t>khóa chính, primary key</t>
+  </si>
+  <si>
+    <t>số định danh, số, id, id khách hàng bên lõi, core banking, mã</t>
+  </si>
+  <si>
+    <t>số, số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch., mã số</t>
+  </si>
+  <si>
+    <t>phân loại tài khoản, ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>đánh dấu tài khoản chính, y/n</t>
+  </si>
+  <si>
+    <t>số, số thứ tự hiển thị tài khoản trên giao diện, app/web, mã số</t>
+  </si>
+  <si>
+    <t>ví dụ: a - active, i - inactive, c - closed, trạng thái tài khoản</t>
+  </si>
+  <si>
+    <t>trạng thái, kết quả, đã xác minh thông tin hay chưa, tình trạng, trạng thái xác thực tài khoản</t>
+  </si>
+  <si>
+    <t>trạng thái kiểm tra, trạng thái, kết quả, mặc định 'u' - unknown hoặc unchecked, tình trạng</t>
+  </si>
+  <si>
+    <t>số định danh, ví dụ: mobile, internet banking, quầy giao dịch, số, id, id kênh tạo tài khoản, mã</t>
+  </si>
+  <si>
+    <t>độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
+  </si>
+  <si>
+    <t>thời gian, ngày, hôm, ngày mở tài khoản hoặc ngày bản ghi được tạo., thời gian, ngày tháng, lịch sử, gần đây</t>
+  </si>
+  <si>
+    <t>tên tài khoản, thường tên chủ tài khoản hoặc tên gợi nhớ, tên, họ tên</t>
+  </si>
+  <si>
+    <t>nơi mở, pgd, mã chi nhánh nơi quản lý tài khoản này., chi nhánh, phòng giao dịch</t>
+  </si>
+  <si>
+    <t>số thẻ được che bớt, ví dụ: 411122****1234</t>
+  </si>
+  <si>
+    <t>customer number, số, mã số khách hàng, mã số</t>
+  </si>
+  <si>
+    <t>số định danh, mã nguồn cung cấp dữ liệu tài khoản này., số, id, mã</t>
+  </si>
+  <si>
+    <t>thời gian, ngày, hôm, ngày hết hạn tài khoản hoặc ngày đóng tài khoản., thời gian, ngày tháng, lịch sử, gần đây</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE id = '{{id}}'"}</t>
@@ -326,7 +379,10 @@
     <t>{"raw_text": "SELECT * FROM customer_account WHERE account_no = '{{account_no}}'"}</t>
   </si>
   <si>
-    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_class = '{{account_class}}'"}</t>
+    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_class = '{{account_class}}' AND check_status = 'SUCCESS'"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer_account WHERE primary_account LIKE '%{{primary_account}}%'"}</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE order_no = '{{order_no}}'"}</t>
@@ -344,9 +400,15 @@
     <t>{"raw_text": "SELECT * FROM customer_account WHERE channel_id = '{{channel_id}}'"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer_account WHERE priority LIKE '%{{priority}}%'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE create_date BETWEEN '{{start_date}}' AND '{{end_date}}' ORDER BY create_date DESC"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_name LIKE '%{{account_name}}%'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE account_branch = '{{account_branch}}'"}</t>
   </si>
   <si>
@@ -360,9 +422,6 @@
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE end_date BETWEEN '{{start_date}}' AND '{{end_date}}' ORDER BY end_date DESC"}</t>
-  </si>
-  <si>
-    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_class = '{{account_class}}' AND create_date BETWEEN '{{start_date}}' AND '{{end_date}}'"}</t>
   </si>
 </sst>
 </file>
@@ -720,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -745,16 +804,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -762,16 +821,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -779,16 +838,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -796,16 +855,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -813,203 +872,237 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
         <v>30</v>
       </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" t="s">
-        <v>62</v>
-      </c>
-      <c r="E17" t="s">
-        <v>78</v>
+      <c r="C19" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E19" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: refine dictionary and adjust faker/generator logic
- Tuned dictionary entries to better align with actual database values
- Improved faker and generator logic to handle cases not explicitly defined in the dictionary
- Enhanced example generation for more realistic and context‑aware outputs
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
   <si>
     <t>document</t>
   </si>
@@ -31,19 +31,19 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu theo khóa chính</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo số định danh</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo số</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo phân loại tài khoản</t>
-  </si>
-  <si>
-    <t>customer_account | Tìm kiếm theo đánh dấu tài khoản chính</t>
+    <t>customer_account | Tra cứu khóa chính</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu id</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch.</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số thứ tự hiển thị tài khoản trên giao diện</t>
   </si>
   <si>
     <t>customer_account | Lọc theo ví dụ: a - active, i - inactive, c - closed</t>
@@ -52,322 +52,261 @@
     <t>customer_account | Lọc theo trạng thái</t>
   </si>
   <si>
-    <t>customer_account | Lọc theo trạng thái kiểm tra</t>
-  </si>
-  <si>
-    <t>customer_account | Tìm kiếm theo độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo thời gian (thời gian)</t>
-  </si>
-  <si>
-    <t>customer_account | Tìm kiếm theo tên tài khoản</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo nơi mở</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo số thẻ được che bớt</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu theo customer number</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên khóa chính (id)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (core_customer_id)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số (account_no)</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách customer_account được phân nhóm bởi phân loại tài khoản. Ví dụ: phân loại tài khoản A, B...</t>
-  </si>
-  <si>
-    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong đánh dấu tài khoản chính</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số (order_no)</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách customer_account được phân nhóm bởi ví dụ: a - active, i - inactive, c - closed. Ví dụ: ví dụ: a - active, i - inactive, c - closed A, B...</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách customer_account được phân nhóm bởi trạng thái. Ví dụ: trạng thái A, B...</t>
-  </si>
-  <si>
-    <t>Liệt kê danh sách customer_account được phân nhóm bởi trạng thái kiểm tra. Ví dụ: trạng thái kiểm tra A, B...</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (channel_id)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử customer_account trong một khoảng thời gian cụ thể (Từ ngày... đến ngày...)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm các customer_account có chứa nội dung/từ khóa trong tên tài khoản</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên nơi mở (account_branch)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số thẻ được che bớt (card_mask)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên customer number (customer_no)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác thông tin customer_account dựa trên số định danh (system_id)</t>
-  </si>
-  <si>
-    <t>Tìm kiếm customer_account ứng với số 913895
-customer_account 560216
-Hãy hiển thị dữ liệu bản ghi customer_account với khóa chính 430935
-Check khóa chính 151612
-Thông tin về customer_account số 193999
-Vui lòng Tra cứu thông tin chi tiết của customer_account có khóa chính là 446305
-Tra cứu customer_account theo khóa chính 296445
-Xem chi tiết 825570
-khóa chính 922006 là của ai?</t>
-  </si>
-  <si>
-    <t>số định danh 127358 là của ai?
-Vui lòng Tra cứu thông tin chi tiết của customer_account có số định danh là 908149
-Thông tin về customer_account số 424316
-Tìm kiếm customer_account ứng với số 227326
-customer_account 704056
-Hãy hiển thị dữ liệu bản ghi customer_account với số định danh 881481
-Xem customer_account theo số định danh 824627
-Xem chi tiết 201516
-Check số định danh 118911</t>
-  </si>
-  <si>
-    <t>Thông tin về customer_account số 416933
-Xem chi tiết 413219
-Check số 655034
-customer_account 381069
-số 523447 là của ai?
-Tìm kiếm customer_account ứng với số 209514
-Hãy hiển thị dữ liệu bản ghi customer_account với số 537525
-Xem customer_account theo số 630521
-Vui lòng Tra cứu thông tin chi tiết của customer_account có số là 124949</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có phân loại tài khoản là hơn
-Tìm tất cả customer_account loại để
-Cho xem danh sách customer_account đã
-Những customer_account nào là cũng?
-Lọc các customer_account đang ở trạng thái đến
-Trích xuất báo cáo các customer_account thuộc loại chưa
-Danh sách vậy</t>
-  </si>
-  <si>
-    <t>Check đánh dấu tài khoản chính từ
-Hãy hiển thị dữ liệu bản ghi customer_account với đánh dấu tài khoản chính đã
-đánh dấu tài khoản chính điều là của ai?
-customer_account nhiều
-Tra cứu customer_account theo đánh dấu tài khoản chính cũng
-Tìm kiếm customer_account ứng với số tự
-Xem chi tiết từ
-Thông tin về customer_account số đã
-Vui lòng Xem thông tin chi tiết của customer_account có đánh dấu tài khoản chính là của</t>
-  </si>
-  <si>
-    <t>Tìm kiếm customer_account ứng với số 386870
-Check số 909408
-Xem customer_account theo số 951122
-Vui lòng Xem thông tin chi tiết của customer_account có số là 277145
-customer_account 329132
-số 534690 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với số 840060
-Xem chi tiết 544336
-Thông tin về customer_account số 440238</t>
-  </si>
-  <si>
-    <t>Những customer_account nào là CŨNG?
-Trích xuất báo cáo các customer_account thuộc loại SỐ
-Tìm tất cả customer_account loại ĐƯỢC
-Lọc các customer_account đang ở trạng thái LỚN
-Hãy liệt kê danh sách các customer_account có ví dụ: a - active, i - inactive, c - closed là CÓ
-customer_account thất bại
-danh sách customer_account thất bại
-Danh sách DƯỚI
-Cho xem danh sách customer_account ĐỂ</t>
-  </si>
-  <si>
-    <t>Tìm tất cả customer_account loại TRONG
-Những customer_account nào là LÀM?
-Cho xem danh sách customer_account NÀY
-danh sách customer_account bị treo
-customer_account bị treo
-Hãy liệt kê danh sách các customer_account có trạng thái là SẼ
-Trích xuất báo cáo các customer_account thuộc loại TẠI
-Lọc các customer_account đang ở trạng thái BÊN
-Danh sách TRONG</t>
-  </si>
-  <si>
-    <t>Những customer_account nào là CŨNG?
-Cho xem danh sách customer_account SAU
-Tìm tất cả customer_account loại CỦA
-customer_account đang chờ
-Lọc các customer_account đang ở trạng thái HƠN
-Hãy liệt kê danh sách các customer_account có trạng thái kiểm tra là THEO
-danh sách customer_account đang chờ
-Danh sách KHIẾN
-Trích xuất báo cáo các customer_account thuộc loại LÀ</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số định danh THẾ
-Thông tin về customer_account số HƠN
-Check số định danh KHÔNG
-Vui lòng Xem thông tin chi tiết của customer_account có số định danh là VỀ
-Tra cứu customer_account theo số định danh VÀI
-số định danh ĐẾN là của ai?
-Tìm kiếm customer_account ứng với số CÓ
-customer_account NHƯ
-Xem chi tiết THẾ</t>
-  </si>
-  <si>
-    <t>Xem customer_account theo độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. trong
-customer_account giống
-Hãy hiển thị dữ liệu bản ghi customer_account với độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. nhiều
-Tìm kiếm customer_account ứng với số vài
-Check độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. thay
-Vui lòng Tra cứu thông tin chi tiết của customer_account có độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. là hơn
-độ ưu tiên tài khoản khi thực hiện các giao dịch tự động. khiến là của ai?
-Xem chi tiết người
-Thông tin về customer_account số là</t>
-  </si>
-  <si>
-    <t>Những customer_account nào diễn ra từ 2026-01-23 đến hôm nay?
-Xem biến động customer_account giữa 2026-01-14 và hôm nay
-Lịch sử customer_account 2026-01-17 đến hôm nay
-Sao kê customer_account từ 2026-01-16 - hôm nay
-Kiểm tra customer_account trong ngày 2026-01-15
-Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-10 đến hôm nay
-Liệt kê các giao dịch phát sinh từ ngày 2026-01-02 tới ngày hôm nay</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với tên tài khoản hơn
-Thông tin về customer_account số có
-Xem chi tiết các
-Tìm kiếm customer_account ứng với số cách
-Xem customer_account theo tên tài khoản lớn
-Vui lòng Tìm thông tin chi tiết của customer_account có tên tài khoản là đến
-Check tên tài khoản nhiều
-customer_account tự
-tên tài khoản hơn là của ai?</t>
-  </si>
-  <si>
-    <t>Vui lòng Tìm thông tin chi tiết của customer_account có nơi mở là vậy
-Check nơi mở lớn
-Xem chi tiết của
-Thông tin về customer_account số đang
-Hãy hiển thị dữ liệu bản ghi customer_account với nơi mở để
-nơi mở sẽ là của ai?
-customer_account bạn
-Tìm kiếm customer_account ứng với số lớn
-Xem customer_account theo nơi mở người</t>
-  </si>
-  <si>
-    <t>Check số thẻ được che bớt rất
-Hãy hiển thị dữ liệu bản ghi customer_account với số thẻ được che bớt các
-Tìm kiếm customer_account ứng với số từng
-Thông tin về customer_account số vì
-Tìm customer_account theo số thẻ được che bớt về
-customer_account giống
-Xem chi tiết tôi
-số thẻ được che bớt theo là của ai?
-Vui lòng Tìm thông tin chi tiết của customer_account có số thẻ được che bớt là cho</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account theo customer number 621908
-Tìm kiếm customer_account ứng với số 541697
-Thông tin về customer_account số 190775
-customer_account 484641
-Vui lòng Xem thông tin chi tiết của customer_account có customer number là 913734
-customer number 904988 là của ai?
-Xem chi tiết 998904
-Check customer number 354129
-Hãy hiển thị dữ liệu bản ghi customer_account với customer number 582931</t>
-  </si>
-  <si>
-    <t>Vui lòng Tra cứu thông tin chi tiết của customer_account có số định danh là 950436
-Tìm kiếm customer_account ứng với số 164102
-Thông tin về customer_account số 724600
-Check số định danh 410234
-Xem chi tiết 436611
-customer_account 824049
-số định danh 410017 là của ai?
-Tra cứu customer_account theo số định danh 389848
-Hãy hiển thị dữ liệu bản ghi customer_account với số định danh 118131</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account từ 2026-01-12 - hôm nay
-Kiểm tra customer_account trong ngày 2026-01-04
-Xem biến động customer_account giữa 2025-12-30 và hôm nay
-Những customer_account nào diễn ra từ 2026-01-03 đến hôm nay?
-Lịch sử customer_account 2026-01-09 đến hôm nay
-Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-13 đến hôm nay
-Liệt kê các giao dịch phát sinh từ ngày 2026-01-05 tới ngày hôm nay</t>
+    <t>customer_account | Tra cứu ví dụ: mobile, internet banking, quầy giao dịch</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian (ngày mở tài khoản hoặc ngày bản ghi được tạo.)</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu phòng giao dịch</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu ví dụ: 411122****1234</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu mã số khách hàng</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian (ngày hết hạn tài khoản hoặc ngày đóng tài khoản.)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo khóa chính (id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo id (core_customer_id)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. (account_no)</t>
+  </si>
+  <si>
+    <t>Liệt kê các giao dịch thuộc nhóm ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo số thứ tự hiển thị tài khoản trên giao diện (order_no)</t>
+  </si>
+  <si>
+    <t>Liệt kê các giao dịch thuộc nhóm ví dụ: a - active, i - inactive, c - closed</t>
+  </si>
+  <si>
+    <t>Liệt kê các giao dịch thuộc nhóm trạng thái</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo ví dụ: mobile, internet banking, quầy giao dịch (channel_id)</t>
+  </si>
+  <si>
+    <t>Xem lịch sử theo ngày mở tài khoản hoặc ngày bản ghi được tạo.</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo phòng giao dịch (account_branch)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo ví dụ: 411122****1234 (card_mask)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo mã số khách hàng (customer_no)</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giao dịch cụ thể theo id (system_id)</t>
+  </si>
+  <si>
+    <t>Xem lịch sử theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản.</t>
+  </si>
+  <si>
+    <t>customer_account 511
+Tìm customer_account theo khóa chính 588
+Thông tin về customer_account số 310
+Xem chi tiết 992
+Tìm kiếm customer_account ứng với số 986
+Check khóa chính 895
+Vui lòng Tra cứu thông tin chi tiết của customer_account có khóa chính là 548
+Hãy hiển thị dữ liệu bản ghi customer_account với khóa chính 711</t>
+  </si>
+  <si>
+    <t>id 3121055 là của ai?
+Xem chi tiết 3021266
+Tìm kiếm customer_account ứng với số 6329368
+customer_account 5818369
+Hãy hiển thị dữ liệu bản ghi customer_account với id 4949419
+Xem customer_account theo id 7803083
+Check id 5697296
+Vui lòng Tìm thông tin chi tiết của customer_account có id là 9283930
+Thông tin về customer_account số 5838556</t>
+  </si>
+  <si>
+    <t>Check số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 287
+Tìm kiếm customer_account ứng với số 665
+customer_account 482
+Thông tin về customer_account số 965
+Xem chi tiết 369
+Vui lòng Kiểm tra thông tin chi tiết của customer_account có số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. là 686
+Kiểm tra customer_account theo số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 746
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch. 231</t>
+  </si>
+  <si>
+    <t>Lọc các customer_account đang ở trạng thái MODE_YLTT
+Danh sách CAT_QLB0
+Trích xuất báo cáo các customer_account thuộc loại CAT_5VLX
+Tìm tất cả customer_account loại MODE_0X1D
+Cho xem danh sách customer_account GRP_046E
+Hãy liệt kê danh sách các customer_account có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... là CAT_VQZC
+Những customer_account nào là TYPE_IN7V?</t>
+  </si>
+  <si>
+    <t>Xem chi tiết 601
+customer_account 935
+Tìm kiếm customer_account ứng với số 266
+Thông tin về customer_account số 295
+Vui lòng Xem thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 859
+Tìm customer_account theo số thứ tự hiển thị tài khoản trên giao diện 796
+Check số thứ tự hiển thị tài khoản trên giao diện 621
+Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị tài khoản trên giao diện 807</t>
+  </si>
+  <si>
+    <t>Tìm tất cả customer_account loại thành công
+customer_account treo
+Hãy liệt kê danh sách các customer_account có ví dụ: a - active, i - inactive, c - closed là lỗi
+Danh sách bị treo
+Những customer_account nào là lỗi?
+liệt kê các customer_account treo
+Trích xuất báo cáo các customer_account thuộc loại lỗi
+Cho xem danh sách customer_account hết hạn
+Lọc các customer_account đang ở trạng thái hoàn tất</t>
+  </si>
+  <si>
+    <t>Tìm tất cả customer_account loại đã xong
+customer_account hết hạn
+Hãy liệt kê danh sách các customer_account có trạng thái là đang chờ
+Trích xuất báo cáo các customer_account thuộc loại thành công
+Những customer_account nào là bị treo?
+Lọc các customer_account đang ở trạng thái lỗi
+Cho xem danh sách customer_account thất bại
+Danh sách quá giờ
+liệt kê các customer_account hết hạn</t>
+  </si>
+  <si>
+    <t>Lọc các customer_account đang ở trạng thái bị treo
+Hãy liệt kê danh sách các customer_account có trạng thái là quá giờ
+Cho xem danh sách customer_account đang chờ
+Danh sách đã xong
+Trích xuất báo cáo các customer_account thuộc loại lỗi
+Những customer_account nào là quá giờ?
+Tìm tất cả customer_account loại xử lý
+customer_account hết hạn
+liệt kê các customer_account hết hạn</t>
+  </si>
+  <si>
+    <t>Vui lòng Tìm thông tin chi tiết của customer_account có ví dụ: mobile, internet banking, quầy giao dịch là internet banking
+customer_account tại quầy
+Thông tin về customer_account số quầy giao dịch
+Kiểm tra customer_account theo ví dụ: mobile, internet banking, quầy giao dịch tại quầy
+Hãy hiển thị dữ liệu bản ghi customer_account với ví dụ: mobile, internet banking, quầy giao dịch tại atm
+Xem chi tiết quầy giao dịch
+Tìm kiếm customer_account ứng với số quầy giao dịch
+Check ví dụ: mobile, internet banking, quầy giao dịch i-banking</t>
+  </si>
+  <si>
+    <t>Kiểm tra customer_account trong ngày 2026-01-24
+Những customer_account nào diễn ra từ 2026-01-21 đến hôm nay?
+Liệt kê các giao dịch phát sinh từ ngày 2025-12-30 tới ngày hôm nay
+Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-09 đến hôm nay
+Xem biến động customer_account giữa 2026-01-02 và hôm nay
+Lịch sử customer_account 2026-01-22 đến hôm nay
+Sao kê customer_account từ 2026-01-09 - hôm nay</t>
+  </si>
+  <si>
+    <t>Tìm kiếm customer_account ứng với số MODE_MSUA
+Thông tin về customer_account số GRP_OWT0
+customer_account CAT_29KE
+Vui lòng Xem thông tin chi tiết của customer_account có phòng giao dịch là MODE_AQRB
+Kiểm tra customer_account theo phòng giao dịch CAT_VK7M
+Hãy hiển thị dữ liệu bản ghi customer_account với phòng giao dịch GRP_80LA
+Check phòng giao dịch CAT_2K2C
+Xem chi tiết TYPE_GUU1</t>
+  </si>
+  <si>
+    <t>Kiểm tra customer_account theo ví dụ: 411122****1234 GRP_4NCG
+Check ví dụ: 411122****1234 GRP_40J5
+Hãy hiển thị dữ liệu bản ghi customer_account với ví dụ: 411122****1234 GRP_JK6A
+Xem chi tiết CAT_GJBS
+Thông tin về customer_account số TYPE_P37P
+Tìm kiếm customer_account ứng với số CAT_BWEF
+customer_account CAT_950U
+Vui lòng Tra cứu thông tin chi tiết của customer_account có ví dụ: 411122****1234 là CAT_7NCX</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với mã số khách hàng 6242308
+Thông tin về customer_account số 1108007
+Check mã số khách hàng 5694753
+mã số khách hàng 3986629 là của ai?
+Tìm kiếm customer_account ứng với số 7436612
+Xem chi tiết 2359622
+Vui lòng Tra cứu thông tin chi tiết của customer_account có mã số khách hàng là 3711919
+customer_account 5908616
+Xem customer_account theo mã số khách hàng 1554561</t>
+  </si>
+  <si>
+    <t>Xem chi tiết 140
+Xem customer_account theo id 829
+Thông tin về customer_account số 905
+customer_account 835
+Vui lòng Tra cứu thông tin chi tiết của customer_account có id là 978
+Hãy hiển thị dữ liệu bản ghi customer_account với id 609
+Check id 656
+Tìm kiếm customer_account ứng với số 488</t>
+  </si>
+  <si>
+    <t>Xem biến động customer_account giữa 2026-01-17 và hôm nay
+Kiểm tra customer_account trong ngày 2026-01-26
+Liệt kê các giao dịch phát sinh từ ngày 2026-01-05 tới ngày hôm nay
+Truy xuất lịch sử customer_account trong khoảng thời gian từ 2026-01-25 đến hôm nay
+Những customer_account nào diễn ra từ 2025-12-30 đến hôm nay?
+Sao kê customer_account từ 2026-01-23 - hôm nay
+Lịch sử customer_account 2026-01-22 đến hôm nay</t>
   </si>
   <si>
     <t>khóa chính, primary key</t>
   </si>
   <si>
-    <t>số định danh, số, id, id khách hàng bên lõi, core banking, mã</t>
-  </si>
-  <si>
-    <t>số, số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch., mã số</t>
-  </si>
-  <si>
-    <t>phân loại tài khoản, ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
-  </si>
-  <si>
-    <t>đánh dấu tài khoản chính, y/n</t>
-  </si>
-  <si>
-    <t>số, số thứ tự hiển thị tài khoản trên giao diện, app/web, mã số</t>
-  </si>
-  <si>
-    <t>ví dụ: a - active, i - inactive, c - closed, trạng thái tài khoản</t>
-  </si>
-  <si>
-    <t>trạng thái, kết quả, đã xác minh thông tin hay chưa, tình trạng, trạng thái xác thực tài khoản</t>
-  </si>
-  <si>
-    <t>trạng thái kiểm tra, trạng thái, kết quả, mặc định 'u' - unknown hoặc unchecked, tình trạng</t>
-  </si>
-  <si>
-    <t>số định danh, ví dụ: mobile, internet banking, quầy giao dịch, số, id, id kênh tạo tài khoản, mã</t>
-  </si>
-  <si>
-    <t>độ ưu tiên tài khoản khi thực hiện các giao dịch tự động.</t>
-  </si>
-  <si>
-    <t>thời gian, ngày, hôm, ngày mở tài khoản hoặc ngày bản ghi được tạo., thời gian, ngày tháng, lịch sử, gần đây</t>
-  </si>
-  <si>
-    <t>tên tài khoản, thường tên chủ tài khoản hoặc tên gợi nhớ, tên, họ tên</t>
-  </si>
-  <si>
-    <t>nơi mở, pgd, mã chi nhánh nơi quản lý tài khoản này., chi nhánh, phòng giao dịch</t>
-  </si>
-  <si>
-    <t>số thẻ được che bớt, ví dụ: 411122****1234</t>
-  </si>
-  <si>
-    <t>customer number, số, mã số khách hàng, mã số</t>
-  </si>
-  <si>
-    <t>số định danh, mã nguồn cung cấp dữ liệu tài khoản này., số, id, mã</t>
-  </si>
-  <si>
-    <t>thời gian, ngày, hôm, ngày hết hạn tài khoản hoặc ngày đóng tài khoản., thời gian, ngày tháng, lịch sử, gần đây</t>
+    <t>id, mã, core banking, số, id khách hàng bên lõi, số định danh</t>
+  </si>
+  <si>
+    <t>số tài khoản hoặc số thẻ. đây thông tin định danh tài khoản giao dịch., số, mã số</t>
+  </si>
+  <si>
+    <t>ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng..., phân loại tài khoản, lọc, danh sách</t>
+  </si>
+  <si>
+    <t>số thứ tự hiển thị tài khoản trên giao diện, số, mã số, app/web</t>
+  </si>
+  <si>
+    <t>ví dụ: a - active, i - inactive, c - closed, trạng thái tài khoản, lọc, danh sách</t>
+  </si>
+  <si>
+    <t>trạng thái, tình trạng, đã xác minh thông tin hay chưa, kết quả, trạng thái xác thực tài khoản, lọc, danh sách</t>
+  </si>
+  <si>
+    <t>trạng thái, trạng thái kiểm tra, tình trạng, kết quả, mặc định 'u' - unknown hoặc unchecked, lọc, danh sách</t>
+  </si>
+  <si>
+    <t>ví dụ: mobile, internet banking, quầy giao dịch, kênh thực hiện, id kênh tạo tài khoản</t>
+  </si>
+  <si>
+    <t>ngày mở tài khoản hoặc ngày bản ghi được tạo., hôm, thời gian, ngày, thời gian</t>
+  </si>
+  <si>
+    <t>phòng giao dịch, nơi mở, mã chi nhánh nơi quản lý tài khoản này., pgd, chi nhánh</t>
+  </si>
+  <si>
+    <t>ví dụ: 411122****1234, số thẻ được che bớt</t>
+  </si>
+  <si>
+    <t>mã số khách hàng, customer number, số, mã số</t>
+  </si>
+  <si>
+    <t>id, mã, mã nguồn cung cấp dữ liệu tài khoản này., số, số định danh</t>
+  </si>
+  <si>
+    <t>ngày hết hạn tài khoản hoặc ngày đóng tài khoản., hôm, thời gian, ngày, thời gian</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE id = '{{id}}'"}</t>
@@ -382,9 +321,6 @@
     <t>{"raw_text": "SELECT * FROM customer_account WHERE account_class = '{{account_class}}' AND check_status = 'SUCCESS'"}</t>
   </si>
   <si>
-    <t>{"raw_text": "SELECT * FROM customer_account WHERE primary_account LIKE '%{{primary_account}}%'"}</t>
-  </si>
-  <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE order_no = '{{order_no}}'"}</t>
   </si>
   <si>
@@ -400,13 +336,7 @@
     <t>{"raw_text": "SELECT * FROM customer_account WHERE channel_id = '{{channel_id}}'"}</t>
   </si>
   <si>
-    <t>{"raw_text": "SELECT * FROM customer_account WHERE priority LIKE '%{{priority}}%'"}</t>
-  </si>
-  <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE create_date BETWEEN '{{start_date}}' AND '{{end_date}}' ORDER BY create_date DESC"}</t>
-  </si>
-  <si>
-    <t>{"raw_text": "SELECT * FROM customer_account WHERE account_name LIKE '%{{account_name}}%'"}</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE account_branch = '{{account_branch}}'"}</t>
@@ -779,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -804,16 +734,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -821,16 +751,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -838,16 +768,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -855,16 +785,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -872,50 +802,50 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -923,16 +853,16 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -940,101 +870,101 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1042,67 +972,16 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" t="s">
-        <v>71</v>
-      </c>
-      <c r="E19" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add dictionary builder for generator module
- Implemented automatic dictionary builder to replace manual dictionary creation
- Streamlined workflow for generator module by reducing repetitive hand-written entries
- Improved scalability and maintainability of example generation logic
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\output\generated_datasets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9628D0CF-DCC4-4329-A29C-9029193D0F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="6343" yWindow="1517" windowWidth="19483" windowHeight="12574" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -31,150 +37,150 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu primary key</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu mã khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo tài khoản loại</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo trạng thái tài khoản</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo verify status</t>
+    <t>customer_account | Tra cứu khóa chính</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu mã core khách hàng</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc theo trạng thái verify</t>
   </si>
   <si>
     <t>customer_account | Lọc theo trạng thái kiểm tra</t>
   </si>
   <si>
-    <t>customer_account | Lọc thời gian theo create date</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo end date</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo primary key</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo mã khách hàng</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo tài khoản loại</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái tài khoản</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo verify status</t>
+    <t>customer_account | Lọc thời gian theo ngày mở tài khoản hoặc ngày bản ghi được tạo.</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu customer number</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản.</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo khóa chính</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo mã core khách hàng</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo trạng thái verify</t>
   </si>
   <si>
     <t>Phân nhóm giao dịch theo trạng thái kiểm tra</t>
   </si>
   <si>
-    <t>Truy vấn lịch sử dựa trên cột create date</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số khách hàng</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột end date</t>
-  </si>
-  <si>
-    <t>Tra cứu customer_account 949 hôm qua
-Kiểm tra lệnh 949
-Xem chi tiết customer_account số 949
-Check giao dịch 949</t>
-  </si>
-  <si>
-    <t>Sao kê cho mã khách hàng 4153363
-Liệt kê giao dịch của khách hàng 4153363
-Xem lịch sử của mã khách hàng 4153363</t>
-  </si>
-  <si>
-    <t>Danh sách customer_account có tài khoản loại là GRP_AC90
-Lọc customer_account theo tài khoản loại GRP_AC90</t>
-  </si>
-  <si>
-    <t>lọc các customer_account đang quá giờ
+    <t>Truy vấn lịch sử dựa trên cột ngày mở tài khoản hoặc ngày bản ghi được tạo.</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo customer number</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày hết hạn tài khoản hoặc ngày đóng tài khoản.</t>
+  </si>
+  <si>
+    <t>Tra cứu customer_account 934 hôm nay
+Xem chi tiết customer_account số 934
+Kiểm tra lệnh 934 đang ở trạng thái nào
+Check giao dịch 934</t>
+  </si>
+  <si>
+    <t>Sao kê cho mã core khách hàng 8883926
+Xem lịch sử của mã core khách hàng 8883926
+Liệt kê giao dịch của khách hàng 8883926</t>
+  </si>
+  <si>
+    <t>Danh sách customer_account có ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... là MODE_13C5
+Lọc customer_account theo ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng... MODE_13C5</t>
+  </si>
+  <si>
+    <t>customer_account thất bại
+lọc các customer_account đang hoàn tất
+customer_account treo
+lọc các customer_account đang thất bại
+customer_account hoàn tất
+lọc các customer_account đang treo
+danh sách customer_account hoàn tất
+danh sách customer_account thất bại
+danh sách customer_account treo</t>
+  </si>
+  <si>
+    <t>customer_account đang chờ
+lọc các customer_account đang lỗi
+danh sách customer_account lỗi
+danh sách customer_account hết hạn
+lọc các customer_account đang đang chờ
+customer_account hết hạn
+customer_account lỗi
+lọc các customer_account đang hết hạn
+danh sách customer_account đang chờ</t>
+  </si>
+  <si>
+    <t>danh sách customer_account đã xong
 customer_account bị treo
-customer_account quá giờ
+lọc các customer_account đang đã xong
 danh sách customer_account treo
-danh sách customer_account quá giờ
 lọc các customer_account đang treo
+customer_account đã xong
 lọc các customer_account đang bị treo
-customer_account treo
-danh sách customer_account bị treo</t>
-  </si>
-  <si>
-    <t>customer_account hoàn tất
-danh sách customer_account hết hạn
-lọc các customer_account đang hết hạn
-danh sách customer_account hoàn tất
-customer_account thất bại
-customer_account hết hạn
-lọc các customer_account đang thất bại
-danh sách customer_account thất bại
-lọc các customer_account đang hoàn tất</t>
-  </si>
-  <si>
-    <t>danh sách customer_account hết hạn
-customer_account đang chờ
-lọc các customer_account đang hết hạn
-lọc các customer_account đang đang chờ
-customer_account thất bại
-customer_account hết hạn
-lọc các customer_account đang thất bại
-danh sách customer_account đang chờ
-danh sách customer_account thất bại</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo create date từ ngày 2025-12-24 đến ngày 2026-01-29
-Lọc customer_account có create date trong khoảng 2025-12-24 - 2026-01-29
-Xem lịch sử customer_account dựa trên create date từ 2025-12-24 tới 2026-01-29
-Kiểm tra các customer_account với create date là ngày 2025-12-24</t>
-  </si>
-  <si>
-    <t>Liệt kê giao dịch của khách hàng 8451483
-Xem lịch sử của số khách hàng 8451483
-Sao kê cho số khách hàng 8451483</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo end date từ ngày 2026-01-11 đến ngày 2026-01-29
-Lọc customer_account có end date trong khoảng 2026-01-11 - 2026-01-29
-Xem lịch sử customer_account dựa trên end date từ 2026-01-11 tới 2026-01-29
-Kiểm tra các customer_account với end date là ngày 2026-01-11</t>
-  </si>
-  <si>
-    <t>primary key</t>
-  </si>
-  <si>
-    <t>mã khách hàng, khách hàng, id khách hàng bên lõi, core banking</t>
-  </si>
-  <si>
-    <t>tài khoản loại, phân loại tài khoản</t>
-  </si>
-  <si>
-    <t>trạng thái tài khoản</t>
-  </si>
-  <si>
-    <t>verify status</t>
-  </si>
-  <si>
-    <t>trạng thái kiểm tra</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, create date</t>
-  </si>
-  <si>
-    <t>số khách hàng, khách hàng, mã số khách hàng, customer number</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, end date</t>
+danh sách customer_account bị treo
+customer_account treo</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo. từ ngày 2026-01-01 đến ngày 2026-02-03
+Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi được tạo. trong khoảng 2026-01-01 - 2026-02-03
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo. từ 2026-01-01 tới 2026-02-03
+Kiểm tra các customer_account với ngày mở tài khoản hoặc ngày bản ghi được tạo. là ngày 2026-01-01</t>
+  </si>
+  <si>
+    <t>Liệt kê giao dịch của khách hàng 3093726
+Sao kê cho customer number 3093726
+Xem lịch sử của customer number 3093726</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản. từ ngày 2025-12-23 đến ngày 2026-02-03
+Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản. trong khoảng 2025-12-23 - 2026-02-03
+Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản. từ 2025-12-23 tới 2026-02-03
+Kiểm tra các customer_account với ngày hết hạn tài khoản hoặc ngày đóng tài khoản. là ngày 2025-12-23</t>
+  </si>
+  <si>
+    <t>khóa chính, primary key, số, mã, id tự tăng, khóa chính, khóa chính định danh duy nhất mỗi bản ghi tài khoản, id tự tăng là khóa chính bản ghi này</t>
+  </si>
+  <si>
+    <t>mã core khách hàng, số core khách hàng, id khách hàng bên lõi map tài khoản với khách hàng, id khách hàng bên lõi, core banking</t>
+  </si>
+  <si>
+    <t>ví dụ: tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng..., loại tài khoản, phân loại tài khoản</t>
+  </si>
+  <si>
+    <t>trạng thái bản ghi, ví dụ: 1-hiệu lực, 0-hết hiệu lực, trạng thái, trạng thái tài khoản, ví dụ: a - active, i - inactive, c - closed</t>
+  </si>
+  <si>
+    <t>trạng thái verify, đã xác minh thông tin hay chưa, trạng thái xác thực tài khoản</t>
+  </si>
+  <si>
+    <t>trạng thái kiểm tra, trạng thái check, mặc định 'u' - unknown hoặc unchecked</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, ngày mở tài khoản hoặc ngày bản ghi được tạo.</t>
+  </si>
+  <si>
+    <t>customer number, mã số khách hàng, số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống, mã số khách hàng với tài khoản</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, ngày hết hạn tài khoản hoặc ngày đóng tài khoản.</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE id = '{{id}}'"}</t>
@@ -207,8 +213,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,10 +266,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -271,13 +280,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -315,7 +332,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -349,6 +366,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -383,9 +401,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -558,11 +577,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="5" width="38.3046875" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,156 +601,156 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" ht="87.45" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(generator): add logic for multi-condition handling
- Implemented support for parsing and generating outputs with multiple filter conditions
- Enhanced generator module to handle complex scenarios beyond single-condition cases
- Improved flexibility and accuracy of rule engine outputs
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
   <si>
     <t>document</t>
   </si>
@@ -31,269 +31,265 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu mã core khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo phân loại tài khoản</t>
+    <t>customer_account | Tra cứu core banking</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số tài khoản</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc tài khoản tiết kiệm</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số trạng thái</t>
   </si>
   <si>
-    <t>customer_account | Lọc theo a - active</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo trạng thái verify</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo trạng thái check</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc theo tên tài khoản</t>
+    <t>customer_account | Lọc trạng thái tài khoản</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày nội dung</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
   </si>
   <si>
     <t>customer_account | Tra cứu tài khoản chi nhánh</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu 411122****1234</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu mã số khách hàng với tài khoản</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo mã core khách hàng</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo phân loại tài khoản</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số trạng thái</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo a - active</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái verify</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái check</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo tên tài khoản</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo tài khoản chi nhánh</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo 411122****1234</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo mã số khách hàng với tài khoản</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
-  </si>
-  <si>
-    <t>Check mã core khách hàng 3619088
-Vui lòng Cho tôi xem thông tin chi tiết của customer_account có mã core khách hàng là 3619088
-Tìm customer_account theo mã core khách hàng 3619088
-Thông tin về customer_account số 3619088
-Hãy hiển thị dữ liệu bản ghi customer_account với mã core khách hàng 3619088
-Xem chi tiết 3619088
-Tìm kiếm customer_account ứng với số 3619088
-Tra cứu mã core khách hàng 3619088 là của ai?
-Cho tôi xem customer_account 3619088</t>
-  </si>
-  <si>
-    <t>Vui lòng Hiển thị thông tin chi tiết của customer_account có số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch là 988
-Tìm kiếm customer_account ứng với số 988
-Xem chi tiết 988
-Liệt kê số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 988 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 988
-Liệt kê customer_account 988
-Thông tin về customer_account số 988
-Tìm customer_account theo số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 988
-Check số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 988</t>
-  </si>
-  <si>
-    <t>Danh sách GRP_FX4U
-Lọc các customer_account đang ở trạng thái GRP_FX4U
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là GRP_FX4U
-Những customer_account nào là GRP_FX4U?
-Cho xem danh sách customer_account GRP_FX4U
-Trích xuất báo cáo các customer_account thuộc loại GRP_FX4U
-Tìm tất cả customer_account loại GRP_FX4U</t>
-  </si>
-  <si>
-    <t>Search customer_account theo số trạng thái 598
-Liệt kê số trạng thái 598 là của ai?
-Tìm kiếm customer_account ứng với số 598
-Cho tôi xem customer_account 598
-Vui lòng Liệt kê thông tin chi tiết của customer_account có số trạng thái là 598
-Xem chi tiết 598
-Check số trạng thái 598
-Thông tin về customer_account số 598
-Hãy hiển thị dữ liệu bản ghi customer_account với số trạng thái 598</t>
-  </si>
-  <si>
-    <t>customer_account thất bại
-Hiển thị danh sách customer_account là thất bại
-Cho xem danh sách customer_account lỗi
-Danh sách lỗi
-customer_account đang chờ
-Hãy liệt kê danh sách các customer_account có a - active là lỗi
-Hiển thị các customer_account thất bại
-customer_account hết hạn
-Những customer_account nào là lỗi?
-Danh sách danh sách customer_account là đang chờ
-Những danh sách customer_account là hết hạn
-Những các customer_account hết hạn
-Tìm tất cả customer_account loại lỗi
-Danh sách các customer_account đang chờ
-Lọc các customer_account đang ở trạng thái lỗi
-Trích xuất báo cáo các customer_account thuộc loại lỗi</t>
-  </si>
-  <si>
-    <t>Tìm tất cả customer_account loại thất bại
-Lọc các các customer_account lỗi
+    <t>customer_account | Tra cứu card mask</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số khách hàng</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo core banking (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số tài khoản (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo tài khoản tiết kiệm</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số trạng thái (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo trạng thái tài khoản</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày nội dung</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo tài khoản chi nhánh (Mã chi nhánh nơi quản lý tài khoản này.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo card mask (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số khách hàng (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
+  </si>
+  <si>
+    <t>Check mã core khách hàng 7206631
+Vui lòng Lọc các thông tin chi tiết của customer_account có mã nội dung khách hàng là 9876469
+Check id khách hàng bên lõi map tài khoản với khách hàng 3487749
+Vui lòng Các thông tin chi tiết của customer_account có số core khách hàng là 9876469
+Các core_customer_id 1638224 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với khách hàng bên lõi 7206631
+Check core banking 6269237
+Hãy hiển thị dữ liệu bản ghi customer_account với số nội dung khách hàng 6269237
+Các core banking 9876469 là của ai?
+Vui lòng Các thông tin chi tiết của customer_account có core banking là 9876469</t>
+  </si>
+  <si>
+    <t>Vui lòng Lọc các thông tin chi tiết của customer_account có số tài khoản số thẻ là 643
+Check số tài khoản 643
+Những số tài khoản 643 là của ai?
+Các customer_account theo số tài khoản số thẻ 755
+Vui lòng Những thông tin chi tiết của customer_account có số tài khoản là 643
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản 422
+Những số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 473 là của ai?
+Các customer_account theo số tài khoản số thẻ 643
+Check số tài khoản số thẻ 473
+Xem chi tiết 643</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account thuộc loại CAT_0S97
+Cho xem danh sách customer_account CAT_MPS7
+Tìm tất cả customer_account loại GRP_0PDT
+Lọc các customer_account đang ở trạng thái CAT_MPS7
+Hãy liệt kê danh sách các customer_account có loại tài khoản là GRP_0PDT
+Tìm tất cả customer_account loại CAT_MPS7
+Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là MODE_P50B
+Cho xem danh sách customer_account MODE_P50B
+Tìm tất cả customer_account loại CAT_0S97
+Hãy liệt kê danh sách các customer_account có account_class là GRP_0PDT</t>
+  </si>
+  <si>
+    <t>Lọc các số order 543 là của ai?
+Check order_no 281
+Các customer_account theo số order 281
+Vui lòng Những thông tin chi tiết của customer_account có số order là 543
+Check số order 385
+Danh sách số thứ tự hiển thị tài khoản trên giao diện 543 là của ai?
+Check số trạng thái 863
+Hãy hiển thị dữ liệu bản ghi customer_account với order_no 359
+Các app/web 385 là của ai?
+Lọc các customer_account theo số order 385</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có trạng thái là hết hạn
+Search danh sách customer_account là đã xong
+Tra cứu các customer_account quá giờ
+Hãy liệt kê danh sách các customer_account có 1-hiệu lực là treo
+Lọc các customer_account đang ở trạng thái hết hạn
+Xem chi tiết các customer_account đã xong
+Hiển thị danh sách customer_account là quá giờ
+Cho xem danh sách customer_account hết hạn
+Kiểm tra danh sách customer_account là đã xong
+Tìm các customer_account lỗi</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account thuộc loại treo
+Lọc các customer_account đang ở trạng thái treo
+Tra cứu danh sách customer_account là đang chờ
+Hãy liệt kê danh sách các customer_account có verify_status là thành công
+Tra cứu danh sách customer_account là hoàn tất
+customer_account quá giờ
+Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là treo
+Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là đã xong
+Liệt kê danh sách customer_account là thất bại
+Cho xem danh sách customer_account lỗi</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có trạng thái check là bị treo
+Liệt kê các customer_account bị treo
+Tìm các customer_account hết hạn
+Trích xuất báo cáo các customer_account thuộc loại hoàn tất
+Hãy liệt kê danh sách các customer_account có trạng thái kiểm tra là hoàn tất
+Xem chi tiết danh sách customer_account là xử lý
 Danh sách thất bại
-customer_account đang chờ
-Lọc các customer_account đang ở trạng thái thất bại
-Cho tôi xem danh sách customer_account là đang chờ
-customer_account hết hạn
-Cho xem danh sách customer_account thất bại
-Những customer_account nào là thất bại?
-Search danh sách customer_account là hết hạn
-Search các customer_account hết hạn
-Lọc các danh sách customer_account là lỗi
-Cho tôi xem các customer_account đang chờ
-Trích xuất báo cáo các customer_account thuộc loại thất bại
-Hãy liệt kê danh sách các customer_account có trạng thái verify là thất bại
-customer_account lỗi</t>
-  </si>
-  <si>
-    <t>customer_account thất bại
-Hiển thị danh sách customer_account là thất bại
-Trích xuất báo cáo các customer_account thuộc loại đang chờ
-Hiển thị các customer_account thành công
-Lọc các customer_account đang ở trạng thái đang chờ
-Những customer_account nào là đang chờ?
-Danh sách đang chờ
-Search danh sách customer_account là treo
-Cho xem danh sách customer_account đang chờ
-Hiển thị các customer_account thất bại
-customer_account treo
-Tìm tất cả customer_account loại đang chờ
-Hãy liệt kê danh sách các customer_account có trạng thái check là đang chờ
-customer_account thành công
-Search các customer_account treo
-Hiển thị danh sách customer_account là thành công</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi tạo từ ngày 2025-12-11 đến ngày 2026-02-05
-Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi tạo trong khoảng 2025-12-11 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi tạo từ 2025-12-11 tới 2026-02-05</t>
-  </si>
-  <si>
-    <t>Những customer_account nào là TYPE_DK0U?
-Hãy liệt kê danh sách các customer_account có tên tài khoản là TYPE_DK0U
-Lọc các customer_account đang ở trạng thái TYPE_DK0U
-Danh sách TYPE_DK0U
-Trích xuất báo cáo các customer_account thuộc loại TYPE_DK0U
-Tìm tất cả customer_account loại TYPE_DK0U
-Cho xem danh sách customer_account TYPE_DK0U</t>
-  </si>
-  <si>
-    <t>Xem chi tiết GRP_2HVS
-Thông tin về customer_account số GRP_2HVS
-Check tài khoản chi nhánh GRP_2HVS
-Kiểm tra customer_account theo tài khoản chi nhánh GRP_2HVS
-Vui lòng Hiển thị thông tin chi tiết của customer_account có tài khoản chi nhánh là GRP_2HVS
-Hiển thị tài khoản chi nhánh GRP_2HVS là của ai?
-Hiển thị customer_account GRP_2HVS
-Tìm kiếm customer_account ứng với số GRP_2HVS
-Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh GRP_2HVS</t>
-  </si>
-  <si>
-    <t>Xem chi tiết MODE_P50U
-Thông tin về customer_account số MODE_P50U
-Vui lòng Tra cứu thông tin chi tiết của customer_account có 411122****1234 là MODE_P50U
-Check 411122****1234 MODE_P50U
-Xem chi tiết customer_account theo 411122****1234 MODE_P50U
-Tìm customer_account MODE_P50U
-Tìm 411122****1234 MODE_P50U là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với 411122****1234 MODE_P50U
-Tìm kiếm customer_account ứng với số MODE_P50U</t>
-  </si>
-  <si>
-    <t>Tìm kiếm customer_account ứng với số 5805769
-Liệt kê customer_account theo mã số khách hàng với tài khoản 5805769
-Xem chi tiết 5805769
-Check mã số khách hàng với tài khoản 5805769
-Thông tin về customer_account số 5805769
-Hãy hiển thị dữ liệu bản ghi customer_account với mã số khách hàng với tài khoản 5805769
-Search mã số khách hàng với tài khoản 5805769 là của ai?
-Vui lòng Search thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 5805769
-Kiểm tra customer_account 5805769</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ ngày 2026-01-18 đến ngày 2026-02-05
-Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-18 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ 2026-01-18 tới 2026-02-05</t>
-  </si>
-  <si>
-    <t>mã core khách hàng, id khách hàng bên lõi map tài khoản với khách hàng, core banking, số nội dung khách hàng, khách hàng bên lõi, mã nội dung khách hàng, số core khách hàng</t>
-  </si>
-  <si>
-    <t>số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản số thẻ, số tài khoản</t>
-  </si>
-  <si>
-    <t>phân loại tài khoản, tài khoản thanh toán, tài khoản tiết kiệm, thẻ tín dụng..., loại tài khoản</t>
-  </si>
-  <si>
-    <t>số trạng thái, số thứ tự hiển thị tài khoản trên giao diện, số order, app/web</t>
-  </si>
-  <si>
-    <t>a - active, i - inactive, trạng thái bản ghi, trạng thái, 1-hiệu lực, c - closed, trạng thái tài khoản, 0-hết hiệu lực</t>
-  </si>
-  <si>
-    <t>trạng thái verify, trạng thái xác thực tài khoản, trạng thái trạng thái, đã xác minh thông tin hay chưa</t>
-  </si>
-  <si>
-    <t>trạng thái check, mặc định là 'u' - unknown hoặc unchecked, trạng thái trạng thái, trạng thái kiểm tra</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>tên tài khoản, thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
-  </si>
-  <si>
-    <t>tài khoản chi nhánh, mã chi nhánh nơi quản lý tài khoản này</t>
-  </si>
-  <si>
-    <t>411122****1234, card mask, số tài khoản mask, số thẻ che bớt để đảm bảo bảo mật</t>
-  </si>
-  <si>
-    <t>mã số khách hàng với tài khoản, mã số khách hàng, customer number, có thể khác với cif tùy theo cấu trúc hệ thống, số khách hàng</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
+customer_account lỗi
+Tìm tất cả customer_account loại hoàn tất
+Hãy liệt kê danh sách các customer_account có trạng thái kiểm tra là bị treo</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account theo create_date từ ngày 2026-01-09 đến ngày 2026-02-05
+Xem lịch sử customer_account dựa trên ngày create từ 2025-12-12 tới 2026-02-05
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi tạo từ 2026-01-20 tới 2026-02-05
+Sao kê customer_account theo ngày create từ ngày 2025-12-27 đến ngày 2026-02-05
+Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi tạo từ ngày 2026-01-20 đến ngày 2026-02-05
+Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi tạo trong khoảng 2026-01-05 - 2026-02-05
+Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi tạo trong khoảng 2025-12-10 - 2026-02-05
+Xem lịch sử customer_account dựa trên create_date từ 2026-01-03 tới 2026-02-05
+Xem lịch sử customer_account dựa trên create_date từ 2026-01-17 tới 2026-02-05
+Sao kê customer_account theo create_date từ ngày 2026-01-21 đến ngày 2026-02-05</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là MODE_LXGO
+Trích xuất báo cáo các customer_account thuộc loại CAT_T4R8
+Danh sách TYPE_JJVV
+Hãy liệt kê danh sách các customer_account có tên tài khoản là TYPE_NIME
+Hãy liệt kê danh sách các customer_account có tên tài khoản là TYPE_JJVV
+Trích xuất báo cáo các customer_account thuộc loại CAT_E8X0
+Lọc các customer_account đang ở trạng thái CAT_T4R8
+Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là CAT_E8X0
+Tìm tất cả customer_account loại MODE_LXGO
+Những customer_account nào là CAT_T4R8?</t>
+  </si>
+  <si>
+    <t>Những customer_account CAT_0W1M
+Lọc các customer_account GRP_ODJO
+Hãy hiển thị dữ liệu bản ghi customer_account với account_branch CAT_9UA8
+Những customer_account GRP_ODJO
+Check account_branch CAT_9UA8
+Lọc các customer_account CAT_0W1M
+Danh sách customer_account CAT_W92V
+Lọc các tài khoản chi nhánh TYPE_VK2T là của ai?
+Xem chi tiết CAT_W92V
+Lọc các customer_account theo tài khoản chi nhánh CAT_W92V</t>
+  </si>
+  <si>
+    <t>Vui lòng Những thông tin chi tiết của customer_account có card mask là CAT_O45N
+Những số tài khoản mask CAT_NM83 là của ai?
+Vui lòng Lọc các thông tin chi tiết của customer_account có card mask là GRP_1SKU
+Check card mask GRP_1SKU
+Vui lòng Những thông tin chi tiết của customer_account có 411122****1234 là TYPE_2RC2
+Những card_mask GRP_HSHC là của ai?
+Check 411122****1234 GRP_HSHC
+Thông tin về customer_account số GRP_HSHC
+Những card_mask CAT_O45N là của ai?
+Những 411122****1234 TYPE_2RC2 là của ai?</t>
+  </si>
+  <si>
+    <t>Vui lòng Những thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 3545050
+Lọc các customer_account theo mã số khách hàng với tài khoản 8451415
+Check customer_no 8328116
+Lọc các customer_account 3545050
+Những customer_account 7269271
+Hãy hiển thị dữ liệu bản ghi customer_account với số khách hàng 7269271
+Hãy hiển thị dữ liệu bản ghi customer_account với có thể khác với cif tùy theo cấu trúc hệ thống 8451415
+Những customer_account theo số khách hàng 7269271
+Danh sách có thể khác với cif tùy theo cấu trúc hệ thống 8451415 là của ai?
+Vui lòng Danh sách thông tin chi tiết của customer_account có số khách hàng là 7269271</t>
+  </si>
+  <si>
+    <t>Lọc customer_account có end_date trong khoảng 2026-01-13 - 2026-02-05
+Sao kê customer_account theo end_date từ ngày 2026-01-17 đến ngày 2026-02-05
+Sao kê customer_account theo end_date từ ngày 2026-01-01 đến ngày 2026-02-05
+Sao kê customer_account theo ngày nội dung từ ngày 2025-12-27 đến ngày 2026-02-05
+Sao kê customer_account theo ngày end từ ngày 2026-01-15 đến ngày 2026-02-05
+Sao kê customer_account theo ngày end từ ngày 2025-12-11 đến ngày 2026-02-05
+Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ 2026-01-21 tới 2026-02-05
+Sao kê customer_account theo ngày nội dung từ ngày 2025-12-11 đến ngày 2026-02-05
+Sao kê customer_account theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ ngày 2025-12-13 đến ngày 2026-02-05
+Sao kê customer_account theo ngày end từ ngày 2026-01-10 đến ngày 2026-02-05</t>
+  </si>
+  <si>
+    <t>core banking, mã core khách hàng, khách hàng bên lõi, số core khách hàng, core_customer_id, id khách hàng bên lõi map tài khoản với khách hàng, số nội dung khách hàng, mã nội dung khách hàng</t>
+  </si>
+  <si>
+    <t>số tài khoản, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản số thẻ, account_no</t>
+  </si>
+  <si>
+    <t>account_class, tài khoản tiết kiệm, tài khoản thanh toán, loại tài khoản, thẻ tín dụng..., phân loại tài khoản</t>
+  </si>
+  <si>
+    <t>số trạng thái, số order, app/web, order_no, số thứ tự hiển thị tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>trạng thái tài khoản, 1-hiệu lực, a - active, status, i - inactive, 0-hết hiệu lực, c - closed, trạng thái, trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>verify_status, đã xác minh thông tin hay chưa, trạng thái trạng thái, trạng thái verify, trạng thái xác thực tài khoản</t>
+  </si>
+  <si>
+    <t>trạng thái check, check_status, trạng thái trạng thái, mặc định là 'u' - unknown hoặc unchecked, trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>ngày nội dung, create_date, ngày create, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
+  </si>
+  <si>
+    <t>account_name, thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản</t>
+  </si>
+  <si>
+    <t>tài khoản chi nhánh, mã chi nhánh nơi quản lý tài khoản này, account_branch</t>
+  </si>
+  <si>
+    <t>411122****1234, số thẻ che bớt để đảm bảo bảo mật, số tài khoản mask, card_mask, card mask</t>
+  </si>
+  <si>
+    <t>số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống, customer_no, mã số khách hàng với tài khoản, mã số khách hàng, customer number</t>
+  </si>
+  <si>
+    <t>ngày nội dung, ngày end, end_date, ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE core_customer_id = '{{core_customer_id}}'"}</t>
@@ -715,16 +711,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -732,16 +728,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -749,16 +745,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -766,16 +762,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -783,16 +779,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -800,135 +796,135 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integrate Vietnamese paraphrase model for example refinement
- Applied chieunq/vietnamese-sentence-paraphase to polish example sentences
- Enhanced fluency and naturalness of generated outputs
- Improved contextual accuracy and readability across generator module
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\output\generated_datasets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649DBEE2-76BE-4A62-8C85-37BD68456FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -31,277 +37,277 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu mã nội dung khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số tài khoản số thẻ</t>
+    <t>customer_account | Tra cứu core banking</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số tài khoản</t>
   </si>
   <si>
     <t>customer_account | Lọc thẻ tín dụng...</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu số thứ tự hiển thị của tài khoản trên giao diện</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc c - closed</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc trạng thái verify</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc tên tài khoản</t>
+    <t>customer_account | Tra cứu số thứ tự hiển thị tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc 1-hiệu lực</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc đã xác minh thông tin hay chưa</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày create</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
   </si>
   <si>
     <t>customer_account | Tra cứu mã chi nhánh nơi quản lý tài khoản này</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu số thẻ che bớt để đảm bảo bảo mật</t>
+    <t>customer_account | Tra cứu số tài khoản mask</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số khách hàng</t>
   </si>
   <si>
-    <t>customer_account | Lọc thời gian theo ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo mã nội dung khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo số tài khoản số thẻ (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
+    <t>customer_account | Lọc thời gian theo ngày nội dung</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo core banking (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số tài khoản (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo thẻ tín dụng...</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo số thứ tự hiển thị của tài khoản trên giao diện (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu theo c - closed</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu theo trạng thái verify</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu theo trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu theo tên tài khoản</t>
+    <t>Tra cứu chính xác theo số thứ tự hiển thị tài khoản trên giao diện (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo 1-hiệu lực</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo đã xác minh thông tin hay chưa</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày create</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo mã chi nhánh nơi quản lý tài khoản này (Mã chi nhánh nơi quản lý tài khoản này.)</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo số thẻ che bớt để đảm bảo bảo mật (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
+    <t>Tra cứu chính xác theo số tài khoản mask (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo số khách hàng (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
   </si>
   <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với id khách hàng bên lõi map tài khoản với khách hàng 6555619
-Lọc các customer_account theo core_customer_id 6555619
-Vui lòng Danh sách thông tin chi tiết của customer_account có mã nội dung khách hàng là 7746060
-Vui lòng Những thông tin chi tiết của customer_account có số core khách hàng là 6555619
-Check mã core khách hàng 7802214
-Tìm kiếm customer_account ứng với số 7746060
-Check core banking 8669876
-Tìm kiếm customer_account ứng với số 8669876
-Những customer_account theo mã nội dung khách hàng 7746060
-Lọc các customer_account 7746060</t>
-  </si>
-  <si>
-    <t>Các số tài khoản hoặc số thẻ 334 là của ai?
-Check số tài khoản hoặc số thẻ 334
-Những customer_account theo số tài khoản số thẻ 745
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ 978
-Những số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 667 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản số thẻ 968
-Danh sách customer_account 334
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ 667
-Những customer_account theo số tài khoản 334
-Vui lòng Những thông tin chi tiết của customer_account có số tài khoản hoặc số thẻ là 968</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có loại tài khoản là GRP_MOX5
-Danh sách MODE_OKN7
-Trích xuất báo cáo các customer_account thuộc loại MODE_OKN7
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là CAT_TIH9
-Cho xem danh sách customer_account CAT_TIH9
-Trích xuất báo cáo các customer_account thuộc loại MODE_IAVN
-Hãy liệt kê danh sách các customer_account có loại tài khoản là MODE_OKN7
-Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là CAT_TIH9
-Hãy liệt kê danh sách các customer_account có account_class là GRP_MOX5
-Cho xem danh sách customer_account GRP_MOX5</t>
-  </si>
-  <si>
-    <t>Vui lòng Những thông tin chi tiết của customer_account có app/web là 374
-Hãy hiển thị dữ liệu bản ghi customer_account với số order 496
-Tìm kiếm customer_account ứng với số 213
-Vui lòng Các thông tin chi tiết của customer_account có số order là 213
-Các customer_account theo app/web 374
-Check số thứ tự hiển thị của tài khoản trên giao diện 374
-Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị của tài khoản trên giao diện 861
-Thông tin về customer_account số 213
-Các số order 374 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với order_no 496</t>
-  </si>
-  <si>
-    <t>Danh sách danh sách customer_account là đã xong
-Lọc các danh sách customer_account là treo
-Search danh sách customer_account là hoàn tất
-Tìm các customer_account đã xong
-Những customer_account nào là thành công?
-Liệt kê các customer_account bị treo
-Danh sách danh sách customer_account là thất bại
-Các danh sách customer_account là lỗi
-Hãy liệt kê danh sách các customer_account có trạng thái là đang chờ
-Tìm tất cả customer_account loại đang chờ</t>
-  </si>
-  <si>
-    <t>Tìm danh sách customer_account là đang chờ
-customer_account bị treo
-Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là lỗi
-Lọc các customer_account đang ở trạng thái đang chờ
-Lọc các customer_account đang ở trạng thái thất bại
-Hãy liệt kê danh sách các customer_account có trạng thái xác thực tài khoản là lỗi
-Tìm tất cả customer_account loại hoàn tất
-Tìm danh sách customer_account là lỗi
-Các danh sách customer_account là hết hạn
-Tìm danh sách customer_account là bị treo</t>
-  </si>
-  <si>
-    <t>Tra cứu danh sách customer_account là thất bại
-Những các customer_account hoàn tất
-Lọc các các customer_account hoàn tất
-Hãy liệt kê danh sách các customer_account có mặc định là 'u' - unknown hoặc unchecked là thành công
-Danh sách đã xong
-Hiển thị danh sách customer_account là treo
-customer_account hoàn tất
-Lọc các các customer_account bị treo
-Lọc các customer_account đang ở trạng thái thành công
-Hãy liệt kê danh sách các customer_account có trạng thái check là đã xong</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo create_date từ ngày 2026-01-03 đến ngày 2026-02-05
-Xem lịch sử customer_account dựa trên create_date từ 2026-01-03 tới 2026-02-05
-Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2025-12-24 tới 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2025-12-21 - 2026-02-05
-Lọc customer_account có create_date trong khoảng 2026-01-08 - 2026-02-05
-Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2025-12-24 đến ngày 2026-02-05
-Lọc customer_account có ngày create trong khoảng 2026-02-01 - 2026-02-05
-Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi tạo trong khoảng 2026-01-03 - 2026-02-05
-Lọc customer_account có create_date trong khoảng 2026-01-04 - 2026-02-05
-Xem lịch sử customer_account dựa trên create_date từ 2025-12-31 tới 2026-02-05</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là CAT_9CXC
-Tìm tất cả customer_account loại GRP_CKK2
-Hãy liệt kê danh sách các customer_account có account_name là CAT_9CXC
-Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là GRP_CKK2
-Lọc các customer_account đang ở trạng thái GRP_C80V
-Hãy liệt kê danh sách các customer_account có account_name là TYPE_850Q
-Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là TYPE_850Q
-Hãy liệt kê danh sách các customer_account có tên tài khoản là GRP_C80V
-Hãy liệt kê danh sách các customer_account có account_name là GRP_CKK2
-Lọc các customer_account đang ở trạng thái GRP_CKK2</t>
-  </si>
-  <si>
-    <t>Các customer_account GRP_US6B
-Check mã chi nhánh nơi quản lý tài khoản này GRP_US6B
-Hãy hiển thị dữ liệu bản ghi customer_account với account_branch CAT_AIOA
-Check tài khoản chi nhánh MODE_O2CR
-Vui lòng Những thông tin chi tiết của customer_account có mã chi nhánh nơi quản lý tài khoản này là TYPE_4AP7
-Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh GRP_US6B
-Những customer_account theo tài khoản chi nhánh GRP_US6B
-Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này TYPE_SN3C
-Check mã chi nhánh nơi quản lý tài khoản này CAT_AIOA
-Các tài khoản chi nhánh GRP_US6B là của ai?</t>
-  </si>
-  <si>
-    <t>Vui lòng Lọc các thông tin chi tiết của customer_account có 411122****1234 là MODE_IH0Z
-Check số tài khoản mask MODE_IH0Z
-Tìm kiếm customer_account ứng với số MODE_IH0Z
-Vui lòng Những thông tin chi tiết của customer_account có số thẻ che bớt để đảm bảo bảo mật là CAT_KM3V
-Những số thẻ được che bớt GRP_PJ8A là của ai?
-Check card mask GRP_142L
-Check số thẻ che bớt để đảm bảo bảo mật CAT_KM3V
-Các customer_account GRP_G3ZA
-Vui lòng Lọc các thông tin chi tiết của customer_account có số thẻ che bớt để đảm bảo bảo mật là MODE_IH0Z
-Thông tin về customer_account số CAT_KM3V</t>
-  </si>
-  <si>
-    <t>Những mã số khách hàng với tài khoản 4088445 là của ai?
-Lọc các customer_account 8778561
-Vui lòng Các thông tin chi tiết của customer_account có số khách hàng là 2459569
-Hãy hiển thị dữ liệu bản ghi customer_account với customer_no 8778561
-Hãy hiển thị dữ liệu bản ghi customer_account với mã số khách hàng với tài khoản 2971072
-Những customer_account theo số khách hàng 4088445
-Hãy hiển thị dữ liệu bản ghi customer_account với có thể khác với cif tùy theo cấu trúc hệ thống 2459569
-Hãy hiển thị dữ liệu bản ghi customer_account với số khách hàng 2971072
-Hãy hiển thị dữ liệu bản ghi customer_account với có thể khác với cif tùy theo cấu trúc hệ thống 8778561
-Lọc các số khách hàng 8778561 là của ai?</t>
-  </si>
-  <si>
-    <t>Lọc customer_account có end_date trong khoảng 2025-12-09 - 2026-02-05
-Sao kê customer_account theo ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ ngày 2025-12-26 đến ngày 2026-02-05
-Sao kê customer_account theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ ngày 2025-12-16 đến ngày 2026-02-05
-Sao kê customer_account theo end_date từ ngày 2025-12-16 đến ngày 2026-02-05
-Xem lịch sử customer_account dựa trên end_date từ 2026-02-01 tới 2026-02-05
-Sao kê customer_account theo ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ ngày 2025-12-28 đến ngày 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2026-01-26 - 2026-02-05
-Sao kê customer_account theo ngày end từ ngày 2025-12-19 đến ngày 2026-02-05
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2025-12-20 tới 2026-02-05
-Lọc customer_account có ngày end trong khoảng 2026-01-31 - 2026-02-05</t>
-  </si>
-  <si>
-    <t>mã nội dung khách hàng, core banking, số nội dung khách hàng, id khách hàng bên lõi map tài khoản với khách hàng, số core khách hàng, khách hàng bên lõi, mã core khách hàng, core_customer_id, id của khách hàng bên hệ thống lõi</t>
-  </si>
-  <si>
-    <t>số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, account_no, số tài khoản, số tài khoản số thẻ, số tài khoản hoặc số thẻ</t>
-  </si>
-  <si>
-    <t>thẻ tín dụng..., tài khoản thanh toán, phân loại tài khoản, loại tài khoản, account_class, tài khoản tiết kiệm</t>
-  </si>
-  <si>
-    <t>số thứ tự hiển thị của tài khoản trên giao diện, số trạng thái, số order, số thứ tự hiển thị tài khoản trên giao diện, app/web, order_no</t>
-  </si>
-  <si>
-    <t>c - closed, 0-hết hiệu lực, i - inactive, trạng thái bản ghi, trạng thái tài khoản, 1-hiệu lực, status, a - active, trạng thái</t>
-  </si>
-  <si>
-    <t>đã xác minh thông tin hay chưa, verify_status, trạng thái verify, trạng thái trạng thái, trạng thái xác thực tài khoản</t>
-  </si>
-  <si>
-    <t>check_status, trạng thái kiểm tra, mặc định là 'u' - unknown hoặc unchecked, trạng thái check, trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày mở tài khoản hoặc ngày bản ghi tạo, ngày nội dung, create_date, ngày create</t>
-  </si>
-  <si>
-    <t>account_name, tên tài khoản, thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
-  </si>
-  <si>
-    <t>account_branch, mã chi nhánh nơi quản lý tài khoản này, tài khoản chi nhánh</t>
-  </si>
-  <si>
-    <t>số thẻ che bớt để đảm bảo bảo mật, card_mask, số tài khoản mask, số thẻ được che bớt, 411122****1234, card mask</t>
-  </si>
-  <si>
-    <t>số khách hàng, mã số khách hàng, mã số khách hàng với tài khoản, có thể khác với cif tùy theo cấu trúc hệ thống, customer_no, customer number</t>
-  </si>
-  <si>
-    <t>end_date, ngày end, ngày nội dung, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản, ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
+    <t>Truy vấn lịch sử dựa trên cột ngày nội dung</t>
+  </si>
+  <si>
+    <t>Các customer_account tuân thủ mã nội dung khách hàng 5118482.
+Vui lòng Truy cập chi tiết của customer_account với số core khách hàng là 5426975.
+Hãy hiển thị dữ liệu bản ghi customer_account với số nội dung khách hàng 5426975
+Danh sách mã core khách hàng 3314067 là của ai?
+Các customer_account theo mã nội dung khách hàng 9279273
+Các customer_account theo mã nội dung khách hàng 5118482
+Danh sách customer_account theo core banking 1093570
+Bạn có thể cho tôi biết tên của các core_customer_id 3314067 không?
+Các core_customer_id 3314067 là của ai?
+Check số core khách hàng 3314067</t>
+  </si>
+  <si>
+    <t>Những customer_account theo số tài khoản hoặc số thẻ 216
+Số tài khoản số thẻ 581 được sử dụng bởi customer_account.
+Danh sách customer_account theo số tài khoản hoặc số thẻ 581
+Lọc các số tài khoản 581 là của ai?
+Lọc các customer_account 216
+Check số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 276
+Vui lòng Các thông tin chi tiết của customer_account có số tài khoản số thẻ là 581
+Check số tài khoản hoặc số thẻ 216
+Định danh tài khoản để giao dịch 276 là số tài khoản hoặc số thẻ.
+Số 276, ngày phát hành cho customer_account.</t>
+  </si>
+  <si>
+    <t>Những customer_account nào là CAT_T8HY?
+Bạn có thể cung cấp danh sách các customer_account có hình thức tài khoản GRP_7EVV không?
+Bạn có thể cung cấp danh sách các customer_account có cùng loại tài khoản MODE_HEDV không?
+Những customer_account nào là CAT_Z7D9?
+Những tổ chức tài chính nào là GRP_7EVV?
+Trích xuất báo cáo các customer_account thuộc loại MODE_HEDV
+Hãy liệt kê danh sách các customer_account có loại tài khoản là GRP_7EVV
+Những tổ chức và tổ chức nào được gọi là GRP_7EVV?
+Cho xem danh sách customer_account CAT_T8HY
+Hãy liệt kê danh sách các customer_account có phân loại tài khoản là GRP_7EVV</t>
+  </si>
+  <si>
+    <t>Vui lòng Các thông tin chi tiết của customer_account có app/web là 450
+Ai là người sáng lập các ứng dụng/web 173?
+Hãy hiển thị dữ liệu bản ghi customer_account với order_no 173
+Vui lòng Danh sách thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 450
+Vui lòng Lọc các thông tin chi tiết của customer_account có order_no là 203
+Lọc các customer_account 450.
+Những customer_account 203
+Các tập tin của bản ghi customer_account với order_no 173 để được hiển thị.
+Các customer_account theo số order 450
+Những ứng dụng/web nào được sử dụng trong các ứng dụng app/web 173?</t>
+  </si>
+  <si>
+    <t>Xác định các cuộc gọi đến một số tài khoản không còn hiệu lực, bao gồm cả các tài khoản hết hạn.
+Hãy liệt kê danh sách các customer_account có a - active là quá giờ
+Một số customer_account sở hữu 1-hiệu lực là quá giờ trong danh sách là gì?
+Hãy liệt kê danh sách các customer_account có 1-hiệu lực là quá giờ
+Kiểm tra các customer_account bị treo
+Các customer_account có quy mô không-hết hiệu lực là gì?
+Xác định các customer_account đã hết hạn.
+Hãy liệt kê danh sách các customer_account có 0-hết hiệu lực là quá giờ
+customer_account lỗi
+Những danh sách customer_account là hết hạn</t>
+  </si>
+  <si>
+    <t>Lọc các customer_account đang ở trạng thái đang chờ
+Liệt kê danh sách customer_account là thành công
+Trích xuất báo cáo các customer_account thuộc loại hết hạn
+Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là đang chờ
+Kiểm tra các customer_account đang chờ xử lý.
+Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là thất bại
+Danh sách các customer_account đã chứng minh thông tin chưa được xác minh là gì?
+Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là treo
+Hãy liệt kê danh sách các customer_account có trạng thái verify là treo
+Quản lý danh sách danh sách customer_account là gì?</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có check_status là hết hạn
+Đánh giá các customer_account đã hoàn thành.
+Lọc các customer_account đang ở trạng thái lỗi
+Hãy liệt kê danh sách các customer_account có mặc định là 'u' - unknown hoặc unchecked là quá giờ
+Những ai là một trong những cá nhân có thể đạt được trạng thái check trong trạng thái chờ, hãy thử xem chúng.
+Các danh sách customer_account là quá giờ
+Phân tích các customer_account đã hoàn thành,
+Có bất kỳ customer_account nào có trạng thái check là đang chờ không?
+Tra cứu danh sách customer_account là hoàn tất
+Việc tìm kiếm danh sách customer_account là kết quả cuối cùng.</t>
+  </si>
+  <si>
+    <t>Ngày nội dung được lọc có sẵn trong khoảng 2026-01-15 - 2026-02-05.
+Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2025-12-29 đến ngày 2026-02-05
+Sao kê customer_account theo ngày create từ ngày 2025-12-16 đến ngày 2026-02-05
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2025-12-11 tới 2026-02-05
+Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi tạo từ ngày 2026-01-26 đến ngày 2026-02-05
+Lọc customer_account có ngày nội dung trong khoảng 2026-01-15 - 2026-02-05
+Từ ngày 2025-12-16 đến ngày 2026-02-05, số liệu thống kê customer_account theo ngày create.
+Từ ngày 2026-01-01 đến ngày 2026-02-05, số liệu của Sao kê customer_account được thiết lập theo ngày mở tài khoản hoặc ngày bản ghi.
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2025-12-18 tới 2026-02-05
+Từ ngày 2026-01-01 đến ngày 2026-02-05, các quy tắc của Sao kê C&amp;A hoặc Ngày phát hành được thiết lập theo ngày mở tài khoản hoặc ngày bản ghi.</t>
+  </si>
+  <si>
+    <t>Xác định các customer_account đang ở trạng thái CAT_JJ6D.
+Trích xuất báo cáo các customer_account thuộc loại GRP_G7MF
+Hãy liệt kê danh sách các customer_account có account_name là GRP_ZISS
+Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là GRP_G7MF
+Một vài ví dụ về các customer_account có account_name là TYPE_DEM7 là gì?
+Lựa chọn các customer_account đang ở trạng thái CAT_JJ6D.
+Có những cá nhân nào cung cấp cho những người có account_name là GRP_ZISS?
+Tôi có thể lấy danh sách các customer_account có tài khoản_name là GRP_ZISS không?
+Lọc các customer_account đang ở trạng thái CAT_JJ6D
+Trích xuất báo cáo các customer_account thuộc loại GRP_ZISS</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này CAT_54OM
+Danh sách customer_account CAT_CNDG
+Bạn có thể cung cấp danh sách các tài khoản chi nhánh GRP_2QZY của bạn?
+Những tài khoản chi nhánh GRP_2QZY là của ai?
+Ai có quyền quản lý tài khoản này CAT_CNDG, và tôi có thể tìm mã chi nhánh tại đây ở đâu?
+Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là CAT_54OM
+Các tài khoản chi nhánh CAT_CNDG là của ai?
+Danh sách account_branch CAT_54OM là của ai?
+Các hồ sơ chi nhánh CAT_CNDG thuộc về ai?
+Ai chịu trách nhiệm quản lý tài khoản CAT_CNDG này?</t>
+  </si>
+  <si>
+    <t>Số tài khoản mask CAT_0Z82 để thấy dữ liệu bản ghi customer_account là gì?
+Danh sách số thẻ che bớt để đảm bảo bảo mật GRP_RPWE là của ai?
+Ai chịu trách nhiệm lọc số thẻ được che giấu TYPE_R0XK?
+Bạn có thể cho tôi biết mã số thẻ được che bớt TYPE_R0XK không?
+Thông tin về customer_account số CAT_9RH3
+Lọc các số thẻ được che bớt TYPE_R0XK là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản mask CAT_0Z82
+Lọc các card mask CAT_0Z82 là của ai?
+Lọc các customer_account theo 411122****1234 CAT_9RH3
+Những 411122****1234 CAT_9RH3 là của ai?</t>
+  </si>
+  <si>
+    <t>Bạn có thể nhớ lại số điện thoại của mình là 2943605 không?
+Số khách hàng 2943605, người điều hành doanh nghiệp của họ là bao nhiêu?
+Hãy hiển thị dữ liệu bản ghi customer_account với số khách hàng 2158370
+Những customer_account theo số khách hàng 2943605
+Các customer_account theo số khách hàng 2158370
+Trích xuất số của các customer_account với mã số khách hàng 1212477.
+Check mã số khách hàng 2158370
+Các customer_account theo mã số khách hàng 2943605
+Check customer number 2943605
+Số khách hàng là 2943605 để xác định các customer_account.</t>
+  </si>
+  <si>
+    <t>Xem lịch sử customer_account dựa trên ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ 2026-01-20 tới 2026-02-05
+Lọc customer_account có ngày end trong khoảng 2026-01-28 - 2026-02-05
+Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ 2025-12-09 tới 2026-02-05
+Ngày hết hạn của các tài khoản hoặc ngày đóng tài khoản do lọc customer_account ghi lại từ ngày 2025-12-09 đến 2026-02-05.
+Ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong đợt tuyển dụng customer_account, 2026-01-20 - 2026-02-05
+Lọc customer_account có ngày end trong khoảng 2025-12-25 - 2026-02-05
+Xem lịch sử customer_account dựa trên ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ 2026-01-27 tới 2026-02-05
+Các nhà tuyển dụng có thể dự kiến sẽ có sự gia tăng trong các năm 2025-12-29, từ 2026-02-05.
+Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản trong khoảng 2025-12-09 - 2026-02-05
+Lọc customer_account có ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-20 - 2026-02-05</t>
+  </si>
+  <si>
+    <t>core banking, số nội dung khách hàng, khách hàng bên lõi, mã nội dung khách hàng, core_customer_id, id khách hàng bên lõi map tài khoản với khách hàng, id của khách hàng bên hệ thống lõi, số core khách hàng, mã core khách hàng</t>
+  </si>
+  <si>
+    <t>số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản, số tài khoản hoặc số thẻ, số tài khoản số thẻ, account_no</t>
+  </si>
+  <si>
+    <t>thẻ tín dụng..., account_class, loại tài khoản, tài khoản thanh toán, phân loại tài khoản, tài khoản tiết kiệm</t>
+  </si>
+  <si>
+    <t>số thứ tự hiển thị tài khoản trên giao diện, số trạng thái, order_no, app/web, số thứ tự hiển thị của tài khoản trên giao diện, số order</t>
+  </si>
+  <si>
+    <t>1-hiệu lực, trạng thái, 0-hết hiệu lực, status, trạng thái tài khoản, c - closed, trạng thái bản ghi, a - active, i - inactive</t>
+  </si>
+  <si>
+    <t>trạng thái trạng thái, trạng thái verify, trạng thái xác thực tài khoản, đã xác minh thông tin hay chưa, verify_status</t>
+  </si>
+  <si>
+    <t>check_status, trạng thái trạng thái, trạng thái check, trạng thái kiểm tra, mặc định là 'u' - unknown hoặc unchecked</t>
+  </si>
+  <si>
+    <t>ngày mở tài khoản hoặc ngày bản ghi tạo, ngày create, ngày nội dung, ngày mở tài khoản hoặc ngày bản ghi được tạo, create_date</t>
+  </si>
+  <si>
+    <t>account_name, thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản</t>
+  </si>
+  <si>
+    <t>account_branch, tài khoản chi nhánh, mã chi nhánh nơi quản lý tài khoản này</t>
+  </si>
+  <si>
+    <t>số tài khoản mask, card mask, 411122****1234, số thẻ được che bớt, số thẻ che bớt để đảm bảo bảo mật, card_mask</t>
+  </si>
+  <si>
+    <t>số khách hàng, mã số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống, mã số khách hàng với tài khoản, customer number, customer_no</t>
+  </si>
+  <si>
+    <t>end_date, ngày end, ngày nội dung, ngày hết hạn tài khoản hoặc ngày đóng tài khoản, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE core_customer_id = '{{core_customer_id}}'"}</t>
@@ -346,8 +352,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,10 +405,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -410,13 +422,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -454,7 +474,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -488,6 +508,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -522,9 +543,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -697,242 +719,246 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="2" width="25" style="3" customWidth="1"/>
+    <col min="3" max="4" width="64.61328125" style="3" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" ht="160.30000000000001" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>45</v>
       </c>
       <c r="E3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" ht="189.45" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>46</v>
       </c>
       <c r="E4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>48</v>
       </c>
       <c r="E6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" ht="204" x14ac:dyDescent="0.4">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" ht="291.45" x14ac:dyDescent="0.4">
+      <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>51</v>
       </c>
       <c r="E9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" ht="204" x14ac:dyDescent="0.4">
+      <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>52</v>
       </c>
       <c r="E10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
+    <row r="11" spans="1:5" ht="189.45" x14ac:dyDescent="0.4">
+      <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
+      <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="3" t="s">
         <v>54</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" ht="160.30000000000001" x14ac:dyDescent="0.4">
+      <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>55</v>
       </c>
       <c r="E13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" ht="262.3" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E14" t="s">

</xml_diff>

<commit_message>
feat(generator): add user name faker and optimize model performance
- Integrated faker logic to generate realistic user names
- Optimized model processing speed for faster response times
- Improved overall efficiency and reliability of generator workflow
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\output\generated_datasets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649DBEE2-76BE-4A62-8C85-37BD68456FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -37,22 +31,22 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu core banking</t>
+    <t>customer_account | Tra cứu id khách hàng bên lõi map tài khoản với khách hàng</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số tài khoản</t>
   </si>
   <si>
-    <t>customer_account | Lọc thẻ tín dụng...</t>
+    <t>customer_account | Lọc phân loại tài khoản</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số thứ tự hiển thị tài khoản trên giao diện</t>
   </si>
   <si>
-    <t>customer_account | Lọc 1-hiệu lực</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc đã xác minh thông tin hay chưa</t>
+    <t>customer_account | Lọc trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc trạng thái verify</t>
   </si>
   <si>
     <t>customer_account | Lọc trạng thái kiểm tra</t>
@@ -61,37 +55,37 @@
     <t>customer_account | Lọc thời gian theo ngày create</t>
   </si>
   <si>
-    <t>customer_account | Lọc thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
+    <t>customer_account | Lọc tên tài khoản</t>
   </si>
   <si>
     <t>customer_account | Tra cứu mã chi nhánh nơi quản lý tài khoản này</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu số tài khoản mask</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày nội dung</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo core banking (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
+    <t>customer_account | Tra cứu số thẻ che bớt để đảm bảo bảo mật</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu mã số khách hàng với tài khoản</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo id khách hàng bên lõi map tài khoản với khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo số tài khoản (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo thẻ tín dụng...</t>
+    <t>Lọc dữ liệu theo phân loại tài khoản</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo số thứ tự hiển thị tài khoản trên giao diện (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo 1-hiệu lực</t>
-  </si>
-  <si>
-    <t>Lọc dữ liệu theo đã xác minh thông tin hay chưa</t>
+    <t>Lọc dữ liệu theo trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>Lọc dữ liệu theo trạng thái verify</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo trạng thái kiểm tra</t>
@@ -100,214 +94,214 @@
     <t>Truy vấn lịch sử dựa trên cột ngày create</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo thường là tên chủ tài khoản hoặc tên gợi nhớ</t>
+    <t>Lọc dữ liệu theo tên tài khoản</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo mã chi nhánh nơi quản lý tài khoản này (Mã chi nhánh nơi quản lý tài khoản này.)</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo số tài khoản mask (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo số khách hàng (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày nội dung</t>
-  </si>
-  <si>
-    <t>Các customer_account tuân thủ mã nội dung khách hàng 5118482.
-Vui lòng Truy cập chi tiết của customer_account với số core khách hàng là 5426975.
-Hãy hiển thị dữ liệu bản ghi customer_account với số nội dung khách hàng 5426975
-Danh sách mã core khách hàng 3314067 là của ai?
-Các customer_account theo mã nội dung khách hàng 9279273
-Các customer_account theo mã nội dung khách hàng 5118482
-Danh sách customer_account theo core banking 1093570
-Bạn có thể cho tôi biết tên của các core_customer_id 3314067 không?
-Các core_customer_id 3314067 là của ai?
-Check số core khách hàng 3314067</t>
-  </si>
-  <si>
-    <t>Những customer_account theo số tài khoản hoặc số thẻ 216
-Số tài khoản số thẻ 581 được sử dụng bởi customer_account.
-Danh sách customer_account theo số tài khoản hoặc số thẻ 581
-Lọc các số tài khoản 581 là của ai?
-Lọc các customer_account 216
-Check số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 276
-Vui lòng Các thông tin chi tiết của customer_account có số tài khoản số thẻ là 581
-Check số tài khoản hoặc số thẻ 216
-Định danh tài khoản để giao dịch 276 là số tài khoản hoặc số thẻ.
-Số 276, ngày phát hành cho customer_account.</t>
-  </si>
-  <si>
-    <t>Những customer_account nào là CAT_T8HY?
-Bạn có thể cung cấp danh sách các customer_account có hình thức tài khoản GRP_7EVV không?
-Bạn có thể cung cấp danh sách các customer_account có cùng loại tài khoản MODE_HEDV không?
-Những customer_account nào là CAT_Z7D9?
-Những tổ chức tài chính nào là GRP_7EVV?
-Trích xuất báo cáo các customer_account thuộc loại MODE_HEDV
-Hãy liệt kê danh sách các customer_account có loại tài khoản là GRP_7EVV
-Những tổ chức và tổ chức nào được gọi là GRP_7EVV?
-Cho xem danh sách customer_account CAT_T8HY
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là GRP_7EVV</t>
-  </si>
-  <si>
-    <t>Vui lòng Các thông tin chi tiết của customer_account có app/web là 450
-Ai là người sáng lập các ứng dụng/web 173?
-Hãy hiển thị dữ liệu bản ghi customer_account với order_no 173
-Vui lòng Danh sách thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 450
-Vui lòng Lọc các thông tin chi tiết của customer_account có order_no là 203
-Lọc các customer_account 450.
-Những customer_account 203
-Các tập tin của bản ghi customer_account với order_no 173 để được hiển thị.
-Các customer_account theo số order 450
-Những ứng dụng/web nào được sử dụng trong các ứng dụng app/web 173?</t>
-  </si>
-  <si>
-    <t>Xác định các cuộc gọi đến một số tài khoản không còn hiệu lực, bao gồm cả các tài khoản hết hạn.
-Hãy liệt kê danh sách các customer_account có a - active là quá giờ
-Một số customer_account sở hữu 1-hiệu lực là quá giờ trong danh sách là gì?
-Hãy liệt kê danh sách các customer_account có 1-hiệu lực là quá giờ
-Kiểm tra các customer_account bị treo
-Các customer_account có quy mô không-hết hiệu lực là gì?
-Xác định các customer_account đã hết hạn.
-Hãy liệt kê danh sách các customer_account có 0-hết hiệu lực là quá giờ
-customer_account lỗi
-Những danh sách customer_account là hết hạn</t>
-  </si>
-  <si>
-    <t>Lọc các customer_account đang ở trạng thái đang chờ
-Liệt kê danh sách customer_account là thành công
-Trích xuất báo cáo các customer_account thuộc loại hết hạn
-Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là đang chờ
-Kiểm tra các customer_account đang chờ xử lý.
-Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là thất bại
-Danh sách các customer_account đã chứng minh thông tin chưa được xác minh là gì?
-Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là treo
-Hãy liệt kê danh sách các customer_account có trạng thái verify là treo
-Quản lý danh sách danh sách customer_account là gì?</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có check_status là hết hạn
-Đánh giá các customer_account đã hoàn thành.
-Lọc các customer_account đang ở trạng thái lỗi
-Hãy liệt kê danh sách các customer_account có mặc định là 'u' - unknown hoặc unchecked là quá giờ
-Những ai là một trong những cá nhân có thể đạt được trạng thái check trong trạng thái chờ, hãy thử xem chúng.
-Các danh sách customer_account là quá giờ
-Phân tích các customer_account đã hoàn thành,
-Có bất kỳ customer_account nào có trạng thái check là đang chờ không?
-Tra cứu danh sách customer_account là hoàn tất
-Việc tìm kiếm danh sách customer_account là kết quả cuối cùng.</t>
-  </si>
-  <si>
-    <t>Ngày nội dung được lọc có sẵn trong khoảng 2026-01-15 - 2026-02-05.
-Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2025-12-29 đến ngày 2026-02-05
-Sao kê customer_account theo ngày create từ ngày 2025-12-16 đến ngày 2026-02-05
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2025-12-11 tới 2026-02-05
-Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi tạo từ ngày 2026-01-26 đến ngày 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2026-01-15 - 2026-02-05
-Từ ngày 2025-12-16 đến ngày 2026-02-05, số liệu thống kê customer_account theo ngày create.
-Từ ngày 2026-01-01 đến ngày 2026-02-05, số liệu của Sao kê customer_account được thiết lập theo ngày mở tài khoản hoặc ngày bản ghi.
-Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2025-12-18 tới 2026-02-05
-Từ ngày 2026-01-01 đến ngày 2026-02-05, các quy tắc của Sao kê C&amp;A hoặc Ngày phát hành được thiết lập theo ngày mở tài khoản hoặc ngày bản ghi.</t>
-  </si>
-  <si>
-    <t>Xác định các customer_account đang ở trạng thái CAT_JJ6D.
-Trích xuất báo cáo các customer_account thuộc loại GRP_G7MF
-Hãy liệt kê danh sách các customer_account có account_name là GRP_ZISS
-Hãy liệt kê danh sách các customer_account có thường là tên chủ tài khoản hoặc tên gợi nhớ là GRP_G7MF
-Một vài ví dụ về các customer_account có account_name là TYPE_DEM7 là gì?
-Lựa chọn các customer_account đang ở trạng thái CAT_JJ6D.
-Có những cá nhân nào cung cấp cho những người có account_name là GRP_ZISS?
-Tôi có thể lấy danh sách các customer_account có tài khoản_name là GRP_ZISS không?
-Lọc các customer_account đang ở trạng thái CAT_JJ6D
-Trích xuất báo cáo các customer_account thuộc loại GRP_ZISS</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này CAT_54OM
-Danh sách customer_account CAT_CNDG
-Bạn có thể cung cấp danh sách các tài khoản chi nhánh GRP_2QZY của bạn?
-Những tài khoản chi nhánh GRP_2QZY là của ai?
-Ai có quyền quản lý tài khoản này CAT_CNDG, và tôi có thể tìm mã chi nhánh tại đây ở đâu?
-Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là CAT_54OM
-Các tài khoản chi nhánh CAT_CNDG là của ai?
-Danh sách account_branch CAT_54OM là của ai?
-Các hồ sơ chi nhánh CAT_CNDG thuộc về ai?
-Ai chịu trách nhiệm quản lý tài khoản CAT_CNDG này?</t>
-  </si>
-  <si>
-    <t>Số tài khoản mask CAT_0Z82 để thấy dữ liệu bản ghi customer_account là gì?
-Danh sách số thẻ che bớt để đảm bảo bảo mật GRP_RPWE là của ai?
-Ai chịu trách nhiệm lọc số thẻ được che giấu TYPE_R0XK?
-Bạn có thể cho tôi biết mã số thẻ được che bớt TYPE_R0XK không?
-Thông tin về customer_account số CAT_9RH3
-Lọc các số thẻ được che bớt TYPE_R0XK là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản mask CAT_0Z82
-Lọc các card mask CAT_0Z82 là của ai?
-Lọc các customer_account theo 411122****1234 CAT_9RH3
-Những 411122****1234 CAT_9RH3 là của ai?</t>
-  </si>
-  <si>
-    <t>Bạn có thể nhớ lại số điện thoại của mình là 2943605 không?
-Số khách hàng 2943605, người điều hành doanh nghiệp của họ là bao nhiêu?
-Hãy hiển thị dữ liệu bản ghi customer_account với số khách hàng 2158370
-Những customer_account theo số khách hàng 2943605
-Các customer_account theo số khách hàng 2158370
-Trích xuất số của các customer_account với mã số khách hàng 1212477.
-Check mã số khách hàng 2158370
-Các customer_account theo mã số khách hàng 2943605
-Check customer number 2943605
-Số khách hàng là 2943605 để xác định các customer_account.</t>
-  </si>
-  <si>
-    <t>Xem lịch sử customer_account dựa trên ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ 2026-01-20 tới 2026-02-05
-Lọc customer_account có ngày end trong khoảng 2026-01-28 - 2026-02-05
+    <t>Tra cứu chính xác theo số thẻ che bớt để đảm bảo bảo mật (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo mã số khách hàng với tài khoản (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 4659165
+Bạn có thể giải thích cách lọc các mã core khách hàng 4659165 không?
+Danh sách customer_account theo khách hàng bên lõi 4880349
+Hãy hiển thị dữ liệu bản ghi customer_account với core banking 4880349
+Check core_customer_id 4880349
+Xem chi tiết 4880349
+Vui lòng Danh sách thông tin chi tiết của customer_account có core banking là 4659165
+Check mã nội dung khách hàng 4659165
+Ai chịu trách nhiệm phân tích các mã core khách hàng 4659165?
+Lọc các customer_account theo số nội dung khách hàng 4163179</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản 661
+Các customer_account theo số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 458
+Vui lòng Lọc các thông tin chi tiết của customer_account có số tài khoản là 458
+Xem chi tiết 458
+Những account_no 458 là của ai?
+Vui lòng kiểm tra các chi tiết cụ thể của customer_account có số tài khoản là 458.
+Lọc các customer_account 661
+Check số tài khoản hoặc số thẻ 661
+Số tài khoản của customer_account với số tài khoản là 458, Vui lòng xem chi tiết của nó.
+Check số tài khoản số thẻ 661</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account thuộc loại 782
+Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 782
+Tìm tất cả customer_account loại 213
+Trích xuất báo cáo các customer_account thuộc loại 213.
+Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là 213
+Trích xuất báo cáo các customer_account thuộc loại 213
+Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 220
+Hãy liệt kê danh sách các customer_account có loại tài khoản là 213
+Hãy liệt kê danh sách các customer_account có loại tài khoản là 782
+Cho xem danh sách customer_account 220</t>
+  </si>
+  <si>
+    <t>Danh sách số order 506 là của ai?
+Danh sách số thứ tự hiển thị tài khoản trên giao diện 506 là của ai?
+Danh sách số thứ tự hiển thị của tài khoản trên giao diện 506 là của ai?
+Check order_no 506
+Các số thứ tự hiển thị tài khoản trên giao diện 524 là của ai?
+Các số thứ tự hiển thị của tài khoản trên giao diện 436 là của ai?
+Những order_no 524 là của ai?
+Lọc các customer_account theo số trạng thái 524
+Kiểm tra số trạng thái 524 của customer_account.
+Vui lòng Lọc các thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 506</t>
+  </si>
+  <si>
+    <t>Các danh sách customer_account là đã xong
+Hiển thị danh sách customer_account là hết hạn
+Hãy liệt kê danh sách các customer_account có a - active là hết hạn
+Hiển thị danh sách customer_account bị treo là gì?
+Tìm tất cả customer_account loại thành công
+Liệt kê các customer_account đã xong
+Những danh sách customer_account là đang chờ
+Hiển thị danh sách customer_account là bị treo
+Danh sách các customer_account treo
+Hiển thị danh sách customer_account là bị treo hoặc bị treo.</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account theo cách treo.
+Những customer_account nào là thành công?
+Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là lỗi
+customer_account thất bại
+Trích xuất báo cáo các customer_account là loại treo.
+Kiểm tra các customer_account treo
+Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là thành công
+Liệt kê các customer_account đang chờ
+customer_account xử lý
+Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là lỗi</t>
+  </si>
+  <si>
+    <t>Những các customer_account lỗi
+Cho tôi xem danh sách customer_account là thất bại
+Hãy liệt kê danh sách các customer_account có check_status là thành công
+Tìm tất cả customer_account loại xử lý
+Có thể truy cập danh sách customer_account đã hoàn thành không?
+Tra cứu các customer_account xử lý
+Lọc các customer_account đang ở trạng thái hoàn tất
+Liệt kê danh sách customer_account là quá giờ
+Cho xem danh sách customer_account xử lý
+Đã hoàn thành việc truy cập danh sách customer_account.</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2025-12-19 đến ngày 2026-02-05
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi tạo từ 2026-01-03 tới 2026-02-05
+Hãy xem lịch sử customer_account dựa trên create_date từ 2026-01-19 đến 2026-02-05.
+Sao kê customer_account theo ngày nội dung từ ngày 2026-01-04 đến ngày 2026-02-05
+Lọc customer_account có create_date trong khoảng 2026-01-25 - 2026-02-05
+Lịch sử customer_account dựa trên create_date từ 2026-01-19 đến 2026-02-05.
+Lọc customer_account có ngày create trong khoảng 2025-12-29 - 2026-02-05
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-02-02 tới 2026-02-05
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2025-12-29 tới 2026-02-05
+Xem lịch sử customer_account dựa trên create_date từ 2026-01-19 tới 2026-02-05</t>
+  </si>
+  <si>
+    <t>Lọc các customer_account đang ở trạng thái Nam Phú Nguyễn
+Tìm tất cả các customer_account loại Cô Vân Phạm.
+Tìm tất cả customer_account loại Nam Phú Nguyễn
+Hãy liệt kê danh sách các customer_account có account_name là Ngọc Đặng
+Truy cập tất cả các customer_account thuộc loại Cô Vân Phạm.
+Tìm tất cả customer_account loại Cô Vân Phạm
+Hãy liệt kê danh sách các customer_account có account_name là Cô Vân Phạm
+Hãy liệt kê danh sách các customer_account có account_name là Nam Phú Nguyễn
+Trích xuất báo cáo các customer_account thuộc loại Nam Phú Nguyễn
+Lọc các customer_account đang ở trạng thái Cô Vân Phạm</t>
+  </si>
+  <si>
+    <t>Vui lòng cung cấp mã chi nhánh nơi quản lý tài khoản 0551206533 cho dữ liệu bản ghi customer_account.
+Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là 0551206533
+Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 6000304725586
+Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 6000304725586
+Mã chi nhánh nơi quản lý tài khoản 0551206533 là cần thiết để hiển thị dữ liệu bản ghi customer_account.
+Xem chi tiết 9807740250105
+Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 0551206533
+Check account_branch 6000304725586
+Check account_branch 9807740250105
+Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 0551206533</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với card mask 45486445562469
+Check card_mask 0350064456
+Vui lòng Danh sách thông tin chi tiết của customer_account có số thẻ được che bớt là 45486445562469
+Tìm kiếm customer_account theo số 45486445562469.
+Hãy hiển thị dữ liệu bản ghi customer_account với số thẻ che bớt để đảm bảo bảo mật 45486445562469
+Số 45486445562469 là số nào cho customer_account?
+Các customer_account 45486445562469
+Tìm kiếm customer_account ứng với số 45486445562469
+Vui lòng Những thông tin chi tiết của customer_account có số thẻ che bớt để đảm bảo bảo mật là 0350064456
+Vui lòng Các thông tin chi tiết của customer_account có số tài khoản mask là 0350064456</t>
+  </si>
+  <si>
+    <t>Có thể tìm thấy customer_account theo số 2154454 không?
+Danh sách customer number 2154454 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với mã số khách hàng với tài khoản 1595687
+Check customer number 7022607
+Tìm kiếm customer_account ứng với số 2154454
+Vui lòng Những thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 2154454
+Các customer_account theo customer number 2154454
+Vui lòng Danh sách thông tin chi tiết của customer_account có customer number là 1595687
+Các customer number 7022607 là của ai?
+Danh sách customer_account theo số khách hàng 7022607</t>
+  </si>
+  <si>
+    <t>Xem lịch sử customer_account dựa trên end_date từ 2025-12-11 tới 2026-02-05
+Lọc customer_account có ngày nội dung trong khoảng 2026-02-03 - 2026-02-05
+Xem lịch sử customer_account dựa trên end_date từ 2026-01-04 đến 2026-02-05.
+Xem lịch sử customer_account dựa trên end_date từ 2026-01-04 tới 2026-02-05
+Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-16 - 2026-02-05
 Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ 2025-12-09 tới 2026-02-05
-Ngày hết hạn của các tài khoản hoặc ngày đóng tài khoản do lọc customer_account ghi lại từ ngày 2025-12-09 đến 2026-02-05.
-Ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong đợt tuyển dụng customer_account, 2026-01-20 - 2026-02-05
-Lọc customer_account có ngày end trong khoảng 2025-12-25 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày hết hạn của tài khoản hoặc ngày đóng tài khoản từ 2026-01-27 tới 2026-02-05
-Các nhà tuyển dụng có thể dự kiến sẽ có sự gia tăng trong các năm 2025-12-29, từ 2026-02-05.
-Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản trong khoảng 2025-12-09 - 2026-02-05
-Lọc customer_account có ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-20 - 2026-02-05</t>
-  </si>
-  <si>
-    <t>core banking, số nội dung khách hàng, khách hàng bên lõi, mã nội dung khách hàng, core_customer_id, id khách hàng bên lõi map tài khoản với khách hàng, id của khách hàng bên hệ thống lõi, số core khách hàng, mã core khách hàng</t>
-  </si>
-  <si>
-    <t>số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản, số tài khoản hoặc số thẻ, số tài khoản số thẻ, account_no</t>
-  </si>
-  <si>
-    <t>thẻ tín dụng..., account_class, loại tài khoản, tài khoản thanh toán, phân loại tài khoản, tài khoản tiết kiệm</t>
-  </si>
-  <si>
-    <t>số thứ tự hiển thị tài khoản trên giao diện, số trạng thái, order_no, app/web, số thứ tự hiển thị của tài khoản trên giao diện, số order</t>
-  </si>
-  <si>
-    <t>1-hiệu lực, trạng thái, 0-hết hiệu lực, status, trạng thái tài khoản, c - closed, trạng thái bản ghi, a - active, i - inactive</t>
-  </si>
-  <si>
-    <t>trạng thái trạng thái, trạng thái verify, trạng thái xác thực tài khoản, đã xác minh thông tin hay chưa, verify_status</t>
-  </si>
-  <si>
-    <t>check_status, trạng thái trạng thái, trạng thái check, trạng thái kiểm tra, mặc định là 'u' - unknown hoặc unchecked</t>
-  </si>
-  <si>
-    <t>ngày mở tài khoản hoặc ngày bản ghi tạo, ngày create, ngày nội dung, ngày mở tài khoản hoặc ngày bản ghi được tạo, create_date</t>
-  </si>
-  <si>
-    <t>account_name, thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản</t>
-  </si>
-  <si>
-    <t>account_branch, tài khoản chi nhánh, mã chi nhánh nơi quản lý tài khoản này</t>
-  </si>
-  <si>
-    <t>số tài khoản mask, card mask, 411122****1234, số thẻ được che bớt, số thẻ che bớt để đảm bảo bảo mật, card_mask</t>
-  </si>
-  <si>
-    <t>số khách hàng, mã số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống, mã số khách hàng với tài khoản, customer number, customer_no</t>
-  </si>
-  <si>
-    <t>end_date, ngày end, ngày nội dung, ngày hết hạn tài khoản hoặc ngày đóng tài khoản, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
+Lọc customer_account có ngày end trong khoảng 2026-02-03 - 2026-02-05
+Lọc customer_account có ngày nội dung trong khoảng 2025-12-15 - 2026-02-05
+Lọc customer_account có ngày nội dung trong khoảng 2026-01-12 - 2026-02-05
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2025-12-15 tới 2026-02-05</t>
+  </si>
+  <si>
+    <t>mã nội dung khách hàng, số nội dung khách hàng, mã core khách hàng, core_customer_id, core banking, id khách hàng bên lõi map tài khoản với khách hàng, khách hàng bên lõi, id của khách hàng bên hệ thống lõi</t>
+  </si>
+  <si>
+    <t>số tài khoản số thẻ, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, account_no, số tài khoản, số tài khoản hoặc số thẻ</t>
+  </si>
+  <si>
+    <t>tài khoản thanh toán, loại tài khoản, phân loại tài khoản, tài khoản tiết kiệm, account_class, thẻ tín dụng...</t>
+  </si>
+  <si>
+    <t>app/web, số trạng thái, số thứ tự hiển thị của tài khoản trên giao diện, order_no, số order, số thứ tự hiển thị tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>trạng thái, a - active, trạng thái bản ghi, i - inactive, c - closed, trạng thái tài khoản, status</t>
+  </si>
+  <si>
+    <t>trạng thái xác thực tài khoản, trạng thái trạng thái, đã xác minh thông tin hay chưa, verify_status, trạng thái verify</t>
+  </si>
+  <si>
+    <t>trạng thái check, mặc định là 'u' - unknown hoặc unchecked, trạng thái kiểm tra, check_status, trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>ngày create, create_date, ngày nội dung, ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
+  </si>
+  <si>
+    <t>tên tài khoản, thường là tên chủ tài khoản hoặc tên gợi nhớ, account_name</t>
+  </si>
+  <si>
+    <t>tài khoản chi nhánh, account_branch, mã chi nhánh nơi quản lý tài khoản này</t>
+  </si>
+  <si>
+    <t>số thẻ che bớt để đảm bảo bảo mật, card mask, card_mask, 411122****1234, số tài khoản mask, số thẻ được che bớt</t>
+  </si>
+  <si>
+    <t>customer number, mã số khách hàng, customer_no, mã số khách hàng với tài khoản, số khách hàng</t>
+  </si>
+  <si>
+    <t>ngày end, ngày nội dung, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản, end_date, ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE core_customer_id = '{{core_customer_id}}'"}</t>
@@ -352,8 +346,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -405,16 +399,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -422,21 +410,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -474,7 +454,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -508,7 +488,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -543,10 +522,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -719,246 +697,242 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="2" width="25" style="3" customWidth="1"/>
-    <col min="3" max="4" width="64.61328125" style="3" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>44</v>
       </c>
       <c r="E2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="160.30000000000001" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>45</v>
       </c>
       <c r="E3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="189.45" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>46</v>
       </c>
       <c r="E4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>47</v>
       </c>
       <c r="E5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>48</v>
       </c>
       <c r="E6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="204" x14ac:dyDescent="0.4">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>49</v>
       </c>
       <c r="E7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" t="s">
         <v>50</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="291.45" x14ac:dyDescent="0.4">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" t="s">
         <v>51</v>
       </c>
       <c r="E9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="204" x14ac:dyDescent="0.4">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" t="s">
         <v>52</v>
       </c>
       <c r="E10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="189.45" x14ac:dyDescent="0.4">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" t="s">
         <v>53</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" t="s">
         <v>54</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="160.30000000000001" x14ac:dyDescent="0.4">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" t="s">
         <v>55</v>
       </c>
       <c r="E13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="262.3" x14ac:dyDescent="0.4">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" t="s">
         <v>56</v>
       </c>
       <c r="E14" t="s">

</xml_diff>

<commit_message>
feat(generator): LoRA fine-tuning and system integration for transaction domain
- Trained T5 model with LoRA on ddq_document dataset (including transaction_history and user_profile document)
- Achieved strong convergence (Validation Loss ~0.002) with excellent understanding of transaction-related queries
- Added LocalParaphraser class in dl_utils.py to load LoRA model and configure low temperature (0.1) for reduced randomness
- Updated generator.py to hybrid approach: Rule-based for structure + AI for fluent phrasing
- Implemented sampling mechanism to select best AI-generated sentences
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -31,277 +31,277 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu id khách hàng bên lõi map tài khoản với khách hàng</t>
+    <t>customer_account | Tra cứu mã core khách hàng</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số tài khoản</t>
   </si>
   <si>
-    <t>customer_account | Lọc phân loại tài khoản</t>
+    <t>customer_account | Lọc loại tài khoản</t>
   </si>
   <si>
     <t>customer_account | Tra cứu số thứ tự hiển thị tài khoản trên giao diện</t>
   </si>
   <si>
-    <t>customer_account | Lọc trạng thái bản ghi</t>
+    <t>customer_account | Lọc trạng thái</t>
   </si>
   <si>
     <t>customer_account | Lọc trạng thái verify</t>
   </si>
   <si>
-    <t>customer_account | Lọc trạng thái kiểm tra</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày create</t>
+    <t>customer_account | Lọc trạng thái check</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày mở tài khoản hoặc ngày bản ghi tạo</t>
   </si>
   <si>
     <t>customer_account | Lọc tên tài khoản</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu mã chi nhánh nơi quản lý tài khoản này</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số thẻ che bớt để đảm bảo bảo mật</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu mã số khách hàng với tài khoản</t>
+    <t>customer_account | Tra cứu tài khoản chi nhánh</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu card mask</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số khách hàng</t>
   </si>
   <si>
     <t>customer_account | Lọc thời gian theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo id khách hàng bên lõi map tài khoản với khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
+    <t>Tra cứu chính xác theo mã core khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo số tài khoản (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo phân loại tài khoản</t>
+    <t>Lọc dữ liệu theo loại tài khoản</t>
   </si>
   <si>
     <t>Tra cứu chính xác theo số thứ tự hiển thị tài khoản trên giao diện (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo trạng thái bản ghi</t>
+    <t>Lọc dữ liệu theo trạng thái</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo trạng thái verify</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo trạng thái kiểm tra</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày create</t>
+    <t>Lọc dữ liệu theo trạng thái check</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày mở tài khoản hoặc ngày bản ghi tạo</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo tên tài khoản</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo mã chi nhánh nơi quản lý tài khoản này (Mã chi nhánh nơi quản lý tài khoản này.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo số thẻ che bớt để đảm bảo bảo mật (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo mã số khách hàng với tài khoản (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
+    <t>Tra cứu chính xác theo tài khoản chi nhánh (Mã chi nhánh nơi quản lý tài khoản này.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo card mask (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số khách hàng (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
   </si>
   <si>
     <t>Truy vấn lịch sử dựa trên cột ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 4659165
-Bạn có thể giải thích cách lọc các mã core khách hàng 4659165 không?
-Danh sách customer_account theo khách hàng bên lõi 4880349
-Hãy hiển thị dữ liệu bản ghi customer_account với core banking 4880349
-Check core_customer_id 4880349
-Xem chi tiết 4880349
-Vui lòng Danh sách thông tin chi tiết của customer_account có core banking là 4659165
-Check mã nội dung khách hàng 4659165
-Ai chịu trách nhiệm phân tích các mã core khách hàng 4659165?
-Lọc các customer_account theo số nội dung khách hàng 4163179</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản 661
-Các customer_account theo số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 458
-Vui lòng Lọc các thông tin chi tiết của customer_account có số tài khoản là 458
-Xem chi tiết 458
-Những account_no 458 là của ai?
-Vui lòng kiểm tra các chi tiết cụ thể của customer_account có số tài khoản là 458.
-Lọc các customer_account 661
-Check số tài khoản hoặc số thẻ 661
-Số tài khoản của customer_account với số tài khoản là 458, Vui lòng xem chi tiết của nó.
-Check số tài khoản số thẻ 661</t>
-  </si>
-  <si>
-    <t>Trích xuất báo cáo các customer_account thuộc loại 782
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 782
-Tìm tất cả customer_account loại 213
-Trích xuất báo cáo các customer_account thuộc loại 213.
-Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là 213
-Trích xuất báo cáo các customer_account thuộc loại 213
-Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 220
-Hãy liệt kê danh sách các customer_account có loại tài khoản là 213
-Hãy liệt kê danh sách các customer_account có loại tài khoản là 782
-Cho xem danh sách customer_account 220</t>
-  </si>
-  <si>
-    <t>Danh sách số order 506 là của ai?
-Danh sách số thứ tự hiển thị tài khoản trên giao diện 506 là của ai?
-Danh sách số thứ tự hiển thị của tài khoản trên giao diện 506 là của ai?
-Check order_no 506
-Các số thứ tự hiển thị tài khoản trên giao diện 524 là của ai?
-Các số thứ tự hiển thị của tài khoản trên giao diện 436 là của ai?
-Những order_no 524 là của ai?
-Lọc các customer_account theo số trạng thái 524
-Kiểm tra số trạng thái 524 của customer_account.
-Vui lòng Lọc các thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 506</t>
-  </si>
-  <si>
-    <t>Các danh sách customer_account là đã xong
-Hiển thị danh sách customer_account là hết hạn
-Hãy liệt kê danh sách các customer_account có a - active là hết hạn
-Hiển thị danh sách customer_account bị treo là gì?
-Tìm tất cả customer_account loại thành công
-Liệt kê các customer_account đã xong
-Những danh sách customer_account là đang chờ
-Hiển thị danh sách customer_account là bị treo
-Danh sách các customer_account treo
-Hiển thị danh sách customer_account là bị treo hoặc bị treo.</t>
-  </si>
-  <si>
-    <t>Trích xuất báo cáo các customer_account theo cách treo.
-Những customer_account nào là thành công?
-Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là lỗi
-customer_account thất bại
-Trích xuất báo cáo các customer_account là loại treo.
-Kiểm tra các customer_account treo
-Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là thành công
+    <t>Check mã nội dung khách hàng 1327995
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã giao dịch hoặc mã tham chiếu.
+Danh sách customer_account 1327995
+Hãy hiển thị dữ liệu bản ghi customer_account với core banking 5758391
+Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 5758391
+Lọc các customer_account 5758391
+Những mã nội dung khách hàng 1327995 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với mã nội dung khách hàng 8011518
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã nguồn cung cấp dịch vụ hoặc mã tham chiếu.
+Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 8011518</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+Check account_no 728
+Danh sách account_no 385 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản 819
+Hãy hiển thị dữ liệu bản ghi customer_account với account_no 819
+Những account_no 819 là của ai?
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nguồn.
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 385</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có thẻ tín dụng... là 486
+Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 486
+Lọc các customer_account đang ở trạng thái 213
+Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 428
+Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là 428
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 213
+Người dùng muốn tra cứu danh sách các giao dịch thanh toán theo số tài khoản nguồn.
+Cho xem danh sách customer_account 213
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị tài khoản trên giao diện 499
+Người dùng muốn tra cứu một tài khoản cụ thể dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
+Vui lòng Các thông tin chi tiết của customer_account có số thứ tự hiển thị của tài khoản trên giao diện là 499
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
+Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị của tài khoản trên giao diện 499
+Lọc các customer_account theo số order 163
+Các app/web 499 là của ai?
+Các customer_account 163
+Các customer_account theo số trạng thái 499
+Vui lòng Những thông tin chi tiết của customer_account có số trạng thái là 163</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+customer_account hết hạn
+Hãy liệt kê danh sách các customer_account có trạng thái tài khoản là thành công
+Xem chi tiết danh sách customer_account là đang chờ
 Liệt kê các customer_account đang chờ
-customer_account xử lý
-Hãy liệt kê danh sách các customer_account có đã xác minh thông tin hay chưa là lỗi</t>
-  </si>
-  <si>
-    <t>Những các customer_account lỗi
-Cho tôi xem danh sách customer_account là thất bại
-Hãy liệt kê danh sách các customer_account có check_status là thành công
-Tìm tất cả customer_account loại xử lý
-Có thể truy cập danh sách customer_account đã hoàn thành không?
-Tra cứu các customer_account xử lý
-Lọc các customer_account đang ở trạng thái hoàn tất
+Danh sách danh sách customer_account là quá giờ
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Trích xuất báo cáo các customer_account thuộc loại thành công
+Lọc các danh sách customer_account là treo</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account thuộc loại đang chờ
+Hãy liệt kê danh sách các customer_account có verify_status là lỗi
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+Hãy liệt kê danh sách các customer_account có trạng thái xác thực tài khoản là quá giờ
+Kiểm tra các customer_account đã xong
+Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là đang chờ
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Hiển thị danh sách customer_account là đã xong
+Cho xem danh sách customer_account lỗi</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có trạng thái check là hoàn tất
 Liệt kê danh sách customer_account là quá giờ
+Cho xem danh sách customer_account hết hạn
+Search các customer_account đã xong
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo danh mục hoặc nhóm tài khoản.
+customer_account hoàn tất
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
 Cho xem danh sách customer_account xử lý
-Đã hoàn thành việc truy cập danh sách customer_account.</t>
-  </si>
-  <si>
-    <t>Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2025-12-19 đến ngày 2026-02-05
-Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi tạo từ 2026-01-03 tới 2026-02-05
-Hãy xem lịch sử customer_account dựa trên create_date từ 2026-01-19 đến 2026-02-05.
-Sao kê customer_account theo ngày nội dung từ ngày 2026-01-04 đến ngày 2026-02-05
-Lọc customer_account có create_date trong khoảng 2026-01-25 - 2026-02-05
-Lịch sử customer_account dựa trên create_date từ 2026-01-19 đến 2026-02-05.
-Lọc customer_account có ngày create trong khoảng 2025-12-29 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-02-02 tới 2026-02-05
-Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2025-12-29 tới 2026-02-05
-Xem lịch sử customer_account dựa trên create_date từ 2026-01-19 tới 2026-02-05</t>
-  </si>
-  <si>
-    <t>Lọc các customer_account đang ở trạng thái Nam Phú Nguyễn
-Tìm tất cả các customer_account loại Cô Vân Phạm.
-Tìm tất cả customer_account loại Nam Phú Nguyễn
-Hãy liệt kê danh sách các customer_account có account_name là Ngọc Đặng
-Truy cập tất cả các customer_account thuộc loại Cô Vân Phạm.
-Tìm tất cả customer_account loại Cô Vân Phạm
-Hãy liệt kê danh sách các customer_account có account_name là Cô Vân Phạm
-Hãy liệt kê danh sách các customer_account có account_name là Nam Phú Nguyễn
-Trích xuất báo cáo các customer_account thuộc loại Nam Phú Nguyễn
-Lọc các customer_account đang ở trạng thái Cô Vân Phạm</t>
-  </si>
-  <si>
-    <t>Vui lòng cung cấp mã chi nhánh nơi quản lý tài khoản 0551206533 cho dữ liệu bản ghi customer_account.
-Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là 0551206533
-Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 6000304725586
-Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 6000304725586
-Mã chi nhánh nơi quản lý tài khoản 0551206533 là cần thiết để hiển thị dữ liệu bản ghi customer_account.
-Xem chi tiết 9807740250105
-Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 0551206533
-Check account_branch 6000304725586
-Check account_branch 9807740250105
-Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 0551206533</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với card mask 45486445562469
-Check card_mask 0350064456
-Vui lòng Danh sách thông tin chi tiết của customer_account có số thẻ được che bớt là 45486445562469
-Tìm kiếm customer_account theo số 45486445562469.
-Hãy hiển thị dữ liệu bản ghi customer_account với số thẻ che bớt để đảm bảo bảo mật 45486445562469
-Số 45486445562469 là số nào cho customer_account?
-Các customer_account 45486445562469
-Tìm kiếm customer_account ứng với số 45486445562469
-Vui lòng Những thông tin chi tiết của customer_account có số thẻ che bớt để đảm bảo bảo mật là 0350064456
-Vui lòng Các thông tin chi tiết của customer_account có số tài khoản mask là 0350064456</t>
-  </si>
-  <si>
-    <t>Có thể tìm thấy customer_account theo số 2154454 không?
-Danh sách customer number 2154454 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với mã số khách hàng với tài khoản 1595687
-Check customer number 7022607
-Tìm kiếm customer_account ứng với số 2154454
-Vui lòng Những thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 2154454
-Các customer_account theo customer number 2154454
-Vui lòng Danh sách thông tin chi tiết của customer_account có customer number là 1595687
-Các customer number 7022607 là của ai?
-Danh sách customer_account theo số khách hàng 7022607</t>
-  </si>
-  <si>
-    <t>Xem lịch sử customer_account dựa trên end_date từ 2025-12-11 tới 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2026-02-03 - 2026-02-05
-Xem lịch sử customer_account dựa trên end_date từ 2026-01-04 đến 2026-02-05.
-Xem lịch sử customer_account dựa trên end_date từ 2026-01-04 tới 2026-02-05
-Lọc customer_account có ngày hết hạn tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-16 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ 2025-12-09 tới 2026-02-05
-Lọc customer_account có ngày end trong khoảng 2026-02-03 - 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2025-12-15 - 2026-02-05
-Lọc customer_account có ngày nội dung trong khoảng 2026-01-12 - 2026-02-05
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2025-12-15 tới 2026-02-05</t>
-  </si>
-  <si>
-    <t>mã nội dung khách hàng, số nội dung khách hàng, mã core khách hàng, core_customer_id, core banking, id khách hàng bên lõi map tài khoản với khách hàng, khách hàng bên lõi, id của khách hàng bên hệ thống lõi</t>
-  </si>
-  <si>
-    <t>số tài khoản số thẻ, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, account_no, số tài khoản, số tài khoản hoặc số thẻ</t>
-  </si>
-  <si>
-    <t>tài khoản thanh toán, loại tài khoản, phân loại tài khoản, tài khoản tiết kiệm, account_class, thẻ tín dụng...</t>
-  </si>
-  <si>
-    <t>app/web, số trạng thái, số thứ tự hiển thị của tài khoản trên giao diện, order_no, số order, số thứ tự hiển thị tài khoản trên giao diện</t>
-  </si>
-  <si>
-    <t>trạng thái, a - active, trạng thái bản ghi, i - inactive, c - closed, trạng thái tài khoản, status</t>
-  </si>
-  <si>
-    <t>trạng thái xác thực tài khoản, trạng thái trạng thái, đã xác minh thông tin hay chưa, verify_status, trạng thái verify</t>
-  </si>
-  <si>
-    <t>trạng thái check, mặc định là 'u' - unknown hoặc unchecked, trạng thái kiểm tra, check_status, trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>ngày create, create_date, ngày nội dung, ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>tên tài khoản, thường là tên chủ tài khoản hoặc tên gợi nhớ, account_name</t>
+Trích xuất báo cáo các customer_account thuộc loại xử lý
+Liệt kê các customer_account quá giờ</t>
+  </si>
+  <si>
+    <t>Lọc customer_account có ngày nội dung trong khoảng 2026-01-27 - 2026-02-06
+Xem lịch sử customer_account dựa trên create_date từ 2025-12-27 tới 2026-02-06
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-27 tới 2026-02-06
+Sao kê customer_account theo ngày create từ ngày 2025-12-20 đến ngày 2026-02-06
+Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi được tạo trong khoảng 2025-12-24 - 2026-02-06
+Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi được tạo trong khoảng 2026-01-08 - 2026-02-06
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo khoảng thời gian xác định.
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã giao dịch hoặc mã tham chiếu.
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã hóa đơn hoặc mã tham chiếu.</t>
+  </si>
+  <si>
+    <t>Lọc các customer_account đang ở trạng thái Hạnh Hữu Trần
+Trích xuất báo cáo các customer_account thuộc loại Bà Bảo Vũ
+Những customer_account nào là Bà Bảo Vũ?
+Những customer_account nào là Ông Hoàng Lê?
+Danh sách Hạnh Hữu Trần
+Người dùng muốn tra cứu danh sách các cá nhân theo trạng thái xử lý hoặc kết quả giao dịch.
+Danh sách Bà Bảo Vũ
+Trích xuất báo cáo các customer_account thuộc loại Hạnh Hữu Trần
+Người dùng muốn tra cứu danh sách những người tham gia giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo danh mục hoặc nhóm sản phẩm.</t>
+  </si>
+  <si>
+    <t>Check account_branch 222722354901
+Check account_branch 98015987542577
+Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 18082129508294
+Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là 98015987542577
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên tài khoản nguồn thực hiện giao dịch.
+Hãy hiển thị dữ liệu bản ghi customer_account với account_branch 222722354901
+Vui lòng Danh sách thông tin chi tiết của customer_account có mã chi nhánh nơi quản lý tài khoản này là 18082129508294
+Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 222722354901
+Check tài khoản chi nhánh 18082129508294
+Danh sách account_branch 222722354901 là của ai?</t>
+  </si>
+  <si>
+    <t>Check card_mask 6163000324789
+Hãy hiển thị dữ liệu bản ghi customer_account với 411122****1234 62390802300
+Lọc các customer_account theo 411122****1234 0566387951021
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản mask 6163000324789
+Hãy hiển thị dữ liệu bản ghi customer_account với card mask 0566387951021
+Lọc các customer_account 6163000324789
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
+Các customer_account theo 411122****1234 6163000324789
+Người dùng muốn tra cứu các giao dịch mua sắm theo số tài khoản nhận tiền hoặc tài khoản đích.
+Check số thẻ được che bớt 0566387951021</t>
+  </si>
+  <si>
+    <t>Danh sách mã số khách hàng 6933679 là của ai?
+Danh sách số khách hàng 4026700 là của ai?
+Người dùng muốn tra cứu danh sách khách hàng của nhà cung cấp dịch vụ theo số tài khoản nguồn.
+Vui lòng Danh sách thông tin chi tiết của customer_account có số khách hàng là 4026700
+Các customer_account theo số khách hàng 7281784
+Các mã số khách hàng 4026700 là của ai?
+Vui lòng Những thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 6933679
+Vui lòng Lọc các thông tin chi tiết của customer_account có customer_no là 7281784
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
+Các mã số khách hàng với tài khoản 6933679 là của ai?</t>
+  </si>
+  <si>
+    <t>Lọc customer_account có ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-28 - 2026-02-06
+Lọc customer_account có end_date trong khoảng 2026-01-29 - 2026-02-06
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-26 tới 2026-02-06
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
+Sao kê customer_account theo ngày end từ ngày 2025-12-22 đến ngày 2026-02-06
+Lọc customer_account có ngày nội dung trong khoảng 2026-01-26 - 2026-02-06
+Xem lịch sử customer_account dựa trên ngày end từ 2025-12-22 tới 2026-02-06
+Sao kê customer_account theo end_date từ ngày 2026-01-29 đến ngày 2026-02-06
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-17 tới 2026-02-06</t>
+  </si>
+  <si>
+    <t>khách hàng bên lõi, số nội dung khách hàng, core_customer_id, mã nội dung khách hàng, id của khách hàng bên hệ thống lõi, core banking, mã core khách hàng, id khách hàng bên lõi map tài khoản với khách hàng</t>
+  </si>
+  <si>
+    <t>account_no, số tài khoản hoặc số thẻ, số tài khoản, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản số thẻ</t>
+  </si>
+  <si>
+    <t>tài khoản tiết kiệm, phân loại tài khoản, account_class, tài khoản thanh toán, thẻ tín dụng..., loại tài khoản</t>
+  </si>
+  <si>
+    <t>số order, order_no, số thứ tự hiển thị tài khoản trên giao diện, số trạng thái, số thứ tự hiển thị của tài khoản trên giao diện, app/web</t>
+  </si>
+  <si>
+    <t>a - active, trạng thái tài khoản, trạng thái, trạng thái bản ghi, status, i - inactive, c - closed</t>
+  </si>
+  <si>
+    <t>đã xác minh thông tin hay chưa, trạng thái verify, verify_status, trạng thái xác thực tài khoản, trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>trạng thái check, check_status, trạng thái kiểm tra, mặc định là 'u' - unknown hoặc unchecked, trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày nội dung, create_date, ngày create, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
+  </si>
+  <si>
+    <t>account_name, thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản</t>
   </si>
   <si>
     <t>tài khoản chi nhánh, account_branch, mã chi nhánh nơi quản lý tài khoản này</t>
   </si>
   <si>
-    <t>số thẻ che bớt để đảm bảo bảo mật, card mask, card_mask, 411122****1234, số tài khoản mask, số thẻ được che bớt</t>
-  </si>
-  <si>
-    <t>customer number, mã số khách hàng, customer_no, mã số khách hàng với tài khoản, số khách hàng</t>
-  </si>
-  <si>
-    <t>ngày end, ngày nội dung, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản, end_date, ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
+    <t>card_mask, số thẻ che bớt để đảm bảo bảo mật, số thẻ được che bớt, số tài khoản mask, card mask, 411122****1234</t>
+  </si>
+  <si>
+    <t>customer number, số khách hàng, customer_no, mã số khách hàng, mã số khách hàng với tài khoản</t>
+  </si>
+  <si>
+    <t>end_date, ngày end, ngày nội dung, ngày hết hạn tài khoản hoặc ngày đóng tài khoản, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE core_customer_id = '{{core_customer_id}}'"}</t>

</xml_diff>

<commit_message>
feat(generate): include getUserProfile data in model retraining
- Added getUserProfile dataset to training pipeline
- Enhanced coverage of user-related intents and profile queries
- Improved model accuracy and contextual understanding in transaction/domain scenarios
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer_account.xlsx
@@ -31,16 +31,16 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu mã core khách hàng</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số tài khoản</t>
+    <t>customer_account | Tra cứu id khách hàng bên lõi map tài khoản với khách hàng</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch</t>
   </si>
   <si>
     <t>customer_account | Lọc loại tài khoản</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu số thứ tự hiển thị tài khoản trên giao diện</t>
+    <t>customer_account | Tra cứu số order</t>
   </si>
   <si>
     <t>customer_account | Lọc trạng thái</t>
@@ -49,10 +49,10 @@
     <t>customer_account | Lọc trạng thái verify</t>
   </si>
   <si>
-    <t>customer_account | Lọc trạng thái check</t>
-  </si>
-  <si>
-    <t>customer_account | Lọc thời gian theo ngày mở tài khoản hoặc ngày bản ghi tạo</t>
+    <t>customer_account | Lọc trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>customer_account | Lọc thời gian theo ngày create</t>
   </si>
   <si>
     <t>customer_account | Lọc tên tài khoản</t>
@@ -61,25 +61,25 @@
     <t>customer_account | Tra cứu tài khoản chi nhánh</t>
   </si>
   <si>
-    <t>customer_account | Tra cứu card mask</t>
-  </si>
-  <si>
-    <t>customer_account | Tra cứu số khách hàng</t>
+    <t>customer_account | Tra cứu số thẻ che bớt để đảm bảo bảo mật</t>
+  </si>
+  <si>
+    <t>customer_account | Tra cứu mã số khách hàng với tài khoản</t>
   </si>
   <si>
     <t>customer_account | Lọc thời gian theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo mã core khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo số tài khoản (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
+    <t>Tra cứu chính xác theo id khách hàng bên lõi map tài khoản với khách hàng (ID của khách hàng bên hệ thống lõi (Core Banking). Dùng để map tài khoản với thông tin khách hàng.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch (Số tài khoản hoặc số thẻ. Đây là thông tin định danh tài khoản để giao dịch.)</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo loại tài khoản</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo số thứ tự hiển thị tài khoản trên giao diện (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
+    <t>Tra cứu chính xác theo số order (Số thứ tự hiển thị của tài khoản trên giao diện (App/Web).)</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo trạng thái</t>
@@ -88,10 +88,10 @@
     <t>Lọc dữ liệu theo trạng thái verify</t>
   </si>
   <si>
-    <t>Lọc dữ liệu theo trạng thái check</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày mở tài khoản hoặc ngày bản ghi tạo</t>
+    <t>Lọc dữ liệu theo trạng thái kiểm tra</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày create</t>
   </si>
   <si>
     <t>Lọc dữ liệu theo tên tài khoản</t>
@@ -100,208 +100,208 @@
     <t>Tra cứu chính xác theo tài khoản chi nhánh (Mã chi nhánh nơi quản lý tài khoản này.)</t>
   </si>
   <si>
-    <t>Tra cứu chính xác theo card mask (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
-  </si>
-  <si>
-    <t>Tra cứu chính xác theo số khách hàng (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
+    <t>Tra cứu chính xác theo số thẻ che bớt để đảm bảo bảo mật (Số thẻ được che bớt (Ví dụ: 411122****1234) để đảm bảo bảo mật thông tin.)</t>
+  </si>
+  <si>
+    <t>Tra cứu chính xác theo mã số khách hàng với tài khoản (Mã số khách hàng (Customer Number) tương ứng với tài khoản.)</t>
   </si>
   <si>
     <t>Truy vấn lịch sử dựa trên cột ngày hết hạn tài khoản hoặc ngày đóng tài khoản</t>
   </si>
   <si>
-    <t>Check mã nội dung khách hàng 1327995
-Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã giao dịch hoặc mã tham chiếu.
-Danh sách customer_account 1327995
-Hãy hiển thị dữ liệu bản ghi customer_account với core banking 5758391
-Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 5758391
-Lọc các customer_account 5758391
-Những mã nội dung khách hàng 1327995 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với mã nội dung khách hàng 8011518
-Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã nguồn cung cấp dịch vụ hoặc mã tham chiếu.
-Hãy hiển thị dữ liệu bản ghi customer_account với core_customer_id 8011518</t>
-  </si>
-  <si>
-    <t>Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+    <t>Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
+Hãy hiển thị dữ liệu bản ghi customer_account với khách hàng bên lõi 4807391
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã khách hàng của nhà cung cấp dịch vụ
+Check số nội dung khách hàng 5592180
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nhận tiền hoặc tài khoản đích.
+Check core banking 4807391
+Lọc các customer_account 4807391
+Hãy hiển thị dữ liệu bản ghi customer_account với id khách hàng bên lõi map tài khoản với khách hàng 4807391
+Hãy hiển thị dữ liệu bản ghi customer_account với id của khách hàng bên hệ thống lõi 5592180
+Hãy hiển thị dữ liệu bản ghi customer_account với mã core khách hàng 4489376</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu các giao dịch mua sắm theo số tài khoản hoặc tài khoản đích.
+Danh sách customer_account theo số tài khoản 781
+Người dùng muốn tra cứu danh sách các giao dịch mua hoặc bán theo trạng thái xử lý hoặc kết quả giao dịch.
+Check số tài khoản 962
+Lọc các số tài khoản hoặc số thẻ 962 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản số thẻ 781
+Các số tài khoản hoặc số thẻ 781 là của ai?
+Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ 781
+Danh sách customer_account 781
+Vui lòng Lọc các thông tin chi tiết của customer_account có số tài khoản hoặc số thẻ là 962</t>
+  </si>
+  <si>
+    <t>Hãy liệt kê danh sách các customer_account có loại tài khoản là 942
+Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là 196
+Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 942
+Cho xem danh sách customer_account 191
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nhận tiền.
+Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 191
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Lọc các customer_account đang ở trạng thái 196
+Những customer_account nào là 191?
+Cho xem danh sách customer_account 942</t>
+  </si>
+  <si>
+    <t>Check số thứ tự hiển thị của tài khoản trên giao diện 964
+Check số order 713
+Người dùng muốn tra cứu lịch sử giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+Vui lòng Danh sách thông tin chi tiết của customer_account có app/web là 713
+Những customer_account theo số trạng thái 655
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
+Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị của tài khoản trên giao diện 655
+Vui lòng Những thông tin chi tiết của customer_account có số thứ tự hiển thị tài khoản trên giao diện là 964
+Xem chi tiết 655
+Check số thứ tự hiển thị tài khoản trên giao diện 655</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+customer_account đã xong
+Hãy liệt kê danh sách các customer_account có c - closed là hoàn tất
+Hãy liệt kê danh sách các customer_account có trạng thái tài khoản là thất bại
+Danh sách thất bại
+Các các customer_account đang chờ
+Kiểm tra danh sách customer_account là quá giờ
+Hiển thị các customer_account quá giờ
+customer_account lỗi
+Cho xem danh sách customer_account hoàn tất</t>
+  </si>
+  <si>
+    <t>customer_account xử lý
+Trích xuất báo cáo các customer_account thuộc loại thất bại
+Lọc các các customer_account thành công
+Hãy liệt kê danh sách các customer_account có trạng thái xác thực tài khoản là hết hạn
+Liệt kê các customer_account hết hạn
+Người dùng muốn tra cứu danh sách các tài khoản theo trạng thái xử lý hoặc kết quả giao dịch.
+Lọc các danh sách customer_account là đã xong
+Hãy liệt kê danh sách các customer_account có trạng thái verify là thành công
+Search các customer_account xử lý
+Người dùng muốn tra cứu danh sách các tài khoản theo trạng thái giao dịch hoặc kết quả giao dịch.</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các customer_account thuộc loại đang chờ
+Tìm tất cả customer_account loại quá giờ
+Những danh sách customer_account là quá giờ
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
+Kiểm tra các customer_account hết hạn
+Hãy liệt kê danh sách các customer_account có trạng thái check là đang chờ
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Những các customer_account quá giờ
+Xem chi tiết các customer_account lỗi
+Các danh sách customer_account là hết hạn</t>
+  </si>
+  <si>
+    <t>Xem lịch sử customer_account dựa trên ngày create từ 2026-01-29 tới 2026-02-09
+Sao kê customer_account theo ngày nội dung từ ngày 2026-02-06 đến ngày 2026-02-09
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+Người dùng muốn tra cứu lịch sử giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
+Sao kê customer_account theo ngày mở tài khoản hoặc ngày bản ghi được tạo từ ngày 2026-02-07 đến ngày 2026-02-09
+Lọc customer_account có ngày create trong khoảng 2025-12-15 - 2026-02-09
+Lọc customer_account có ngày nội dung trong khoảng 2026-01-09 - 2026-02-09
+Xem lịch sử customer_account dựa trên create_date từ 2026-01-03 tới 2026-02-09
+Xem lịch sử customer_account dựa trên ngày mở tài khoản hoặc ngày bản ghi được tạo từ 2026-01-26 tới 2026-02-09
+Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-08 tới 2026-02-09</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo danh mục hoặc nhóm sản phẩm.
+Hãy liệt kê danh sách các customer_account có account_name là Nhật Hữu Vũ
+Những customer_account nào là Bà Chi Đặng?
+Danh sách Minh Phú Nguyễn
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo tên người dùng muốn tra cứu.
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo tên người dùng muốn tra cứu hoặc kết quả giao dịch.
+Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
+Tìm tất cả customer_account loại Bà Chi Đặng
+Cho xem danh sách customer_account Nhật Hữu Vũ
+Lọc các customer_account đang ở trạng thái Nhật Hữu Vũ</t>
+  </si>
+  <si>
+    <t>Những customer_account theo account_branch 94948155749649
+Lọc các customer_account theo tài khoản chi nhánh 39570257230
+Các account_branch 94948155749649 là của ai?
+Vui lòng Danh sách thông tin chi tiết của customer_account có account_branch là 9164894957464
+Các customer_account 94948155749649
+Danh sách account_branch 39570257230 là của ai?
+Những mã chi nhánh nơi quản lý tài khoản này 94948155749649 là của ai?
+Người dùng muốn tra cứu một tài khoản cụ thể dựa trên mã nguồn cấp dữ liệu hoặc mã tham chiếu.
+Người dùng muốn tra cứu một tài khoản cụ thể dựa trên mã tài khoản nguồn thực hiện giao dịch.
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nhận tiền hoặc tài khoản đích.</t>
+  </si>
+  <si>
+    <t>Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã giao dịch hoặc mã tham chiếu.
+Hãy hiển thị dữ liệu bản ghi customer_account với card mask 5537954565
+Người dùng muốn tra cứu thông tin giao dịch hoặc mã hóa đơn theo số tài khoản nguồn.
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
+Những customer_account theo số tài khoản mask 5537954565
+Xem chi tiết 01950337952800
+Lọc các customer_account theo card_mask 01950337952800
+Hãy hiển thị dữ liệu bản ghi customer_account với 411122****1234 5537954565
+Check 411122****1234 01950337952800
+Xem chi tiết 5537954565</t>
+  </si>
+  <si>
+    <t>Các customer number 6981595 là của ai?
+Các mã số khách hàng với tài khoản 6981595 là của ai?
+Vui lòng Danh sách thông tin chi tiết của customer_account có số khách hàng là 4649107
+Xem chi tiết 6981595
+Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
+Hãy hiển thị dữ liệu bản ghi customer_account với customer_no 5456929
+Những mã số khách hàng với tài khoản 5456929 là của ai?
+Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
 Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
-Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nguồn.
-Check account_no 728
-Danh sách account_no 385 là của ai?
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản 819
-Hãy hiển thị dữ liệu bản ghi customer_account với account_no 819
-Những account_no 819 là của ai?
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nguồn.
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch 385</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có thẻ tín dụng... là 486
-Hãy liệt kê danh sách các customer_account có tài khoản thanh toán là 486
-Lọc các customer_account đang ở trạng thái 213
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 428
-Hãy liệt kê danh sách các customer_account có tài khoản tiết kiệm là 428
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
-Hãy liệt kê danh sách các customer_account có phân loại tài khoản là 213
-Người dùng muốn tra cứu danh sách các giao dịch thanh toán theo số tài khoản nguồn.
-Cho xem danh sách customer_account 213
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.</t>
-  </si>
-  <si>
-    <t>Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị tài khoản trên giao diện 499
-Người dùng muốn tra cứu một tài khoản cụ thể dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
-Vui lòng Các thông tin chi tiết của customer_account có số thứ tự hiển thị của tài khoản trên giao diện là 499
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
-Hãy hiển thị dữ liệu bản ghi customer_account với số thứ tự hiển thị của tài khoản trên giao diện 499
-Lọc các customer_account theo số order 163
-Các app/web 499 là của ai?
-Các customer_account 163
-Các customer_account theo số trạng thái 499
-Vui lòng Những thông tin chi tiết của customer_account có số trạng thái là 163</t>
-  </si>
-  <si>
-    <t>Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
-Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
-customer_account hết hạn
-Hãy liệt kê danh sách các customer_account có trạng thái tài khoản là thành công
-Xem chi tiết danh sách customer_account là đang chờ
-Liệt kê các customer_account đang chờ
-Danh sách danh sách customer_account là quá giờ
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
-Trích xuất báo cáo các customer_account thuộc loại thành công
-Lọc các danh sách customer_account là treo</t>
-  </si>
-  <si>
-    <t>Trích xuất báo cáo các customer_account thuộc loại đang chờ
-Hãy liệt kê danh sách các customer_account có verify_status là lỗi
-Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo trạng thái xử lý hoặc kết quả giao dịch.
-Hãy liệt kê danh sách các customer_account có trạng thái xác thực tài khoản là quá giờ
-Kiểm tra các customer_account đã xong
-Hãy liệt kê danh sách các customer_account có trạng thái trạng thái là đang chờ
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
-Hiển thị danh sách customer_account là đã xong
-Cho xem danh sách customer_account lỗi</t>
-  </si>
-  <si>
-    <t>Hãy liệt kê danh sách các customer_account có trạng thái check là hoàn tất
-Liệt kê danh sách customer_account là quá giờ
-Cho xem danh sách customer_account hết hạn
-Search các customer_account đã xong
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo danh mục hoặc nhóm tài khoản.
-customer_account hoàn tất
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
-Cho xem danh sách customer_account xử lý
-Trích xuất báo cáo các customer_account thuộc loại xử lý
-Liệt kê các customer_account quá giờ</t>
-  </si>
-  <si>
-    <t>Lọc customer_account có ngày nội dung trong khoảng 2026-01-27 - 2026-02-06
-Xem lịch sử customer_account dựa trên create_date từ 2025-12-27 tới 2026-02-06
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-27 tới 2026-02-06
-Sao kê customer_account theo ngày create từ ngày 2025-12-20 đến ngày 2026-02-06
-Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi được tạo trong khoảng 2025-12-24 - 2026-02-06
-Lọc customer_account có ngày mở tài khoản hoặc ngày bản ghi được tạo trong khoảng 2026-01-08 - 2026-02-06
+Những mã số khách hàng 5456929 là của ai?</t>
+  </si>
+  <si>
+    <t>Sao kê customer_account theo ngày hết hạn tài khoản hoặc ngày đóng tài khoản từ ngày 2026-01-16 đến ngày 2026-02-09
+Xem lịch sử customer_account dựa trên end_date từ 2026-01-11 tới 2026-02-09
 Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo khoảng thời gian xác định.
-Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã giao dịch hoặc mã tham chiếu.
-Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã hóa đơn hoặc mã tham chiếu.</t>
-  </si>
-  <si>
-    <t>Lọc các customer_account đang ở trạng thái Hạnh Hữu Trần
-Trích xuất báo cáo các customer_account thuộc loại Bà Bảo Vũ
-Những customer_account nào là Bà Bảo Vũ?
-Những customer_account nào là Ông Hoàng Lê?
-Danh sách Hạnh Hữu Trần
-Người dùng muốn tra cứu danh sách các cá nhân theo trạng thái xử lý hoặc kết quả giao dịch.
-Danh sách Bà Bảo Vũ
-Trích xuất báo cáo các customer_account thuộc loại Hạnh Hữu Trần
-Người dùng muốn tra cứu danh sách những người tham gia giao dịch mua sắm theo trạng thái xử lý hoặc kết quả giao dịch.
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo danh mục hoặc nhóm sản phẩm.</t>
-  </si>
-  <si>
-    <t>Check account_branch 222722354901
-Check account_branch 98015987542577
-Hãy hiển thị dữ liệu bản ghi customer_account với tài khoản chi nhánh 18082129508294
-Vui lòng Danh sách thông tin chi tiết của customer_account có tài khoản chi nhánh là 98015987542577
-Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên tài khoản nguồn thực hiện giao dịch.
-Hãy hiển thị dữ liệu bản ghi customer_account với account_branch 222722354901
-Vui lòng Danh sách thông tin chi tiết của customer_account có mã chi nhánh nơi quản lý tài khoản này là 18082129508294
-Hãy hiển thị dữ liệu bản ghi customer_account với mã chi nhánh nơi quản lý tài khoản này 222722354901
-Check tài khoản chi nhánh 18082129508294
-Danh sách account_branch 222722354901 là của ai?</t>
-  </si>
-  <si>
-    <t>Check card_mask 6163000324789
-Hãy hiển thị dữ liệu bản ghi customer_account với 411122****1234 62390802300
-Lọc các customer_account theo 411122****1234 0566387951021
-Hãy hiển thị dữ liệu bản ghi customer_account với số tài khoản mask 6163000324789
-Hãy hiển thị dữ liệu bản ghi customer_account với card mask 0566387951021
-Lọc các customer_account 6163000324789
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền dựa trên số tài khoản nhận tiền hoặc tài khoản đích.
-Các customer_account theo 411122****1234 6163000324789
-Người dùng muốn tra cứu các giao dịch mua sắm theo số tài khoản nhận tiền hoặc tài khoản đích.
-Check số thẻ được che bớt 0566387951021</t>
-  </si>
-  <si>
-    <t>Danh sách mã số khách hàng 6933679 là của ai?
-Danh sách số khách hàng 4026700 là của ai?
-Người dùng muốn tra cứu danh sách khách hàng của nhà cung cấp dịch vụ theo số tài khoản nguồn.
-Vui lòng Danh sách thông tin chi tiết của customer_account có số khách hàng là 4026700
-Các customer_account theo số khách hàng 7281784
-Các mã số khách hàng 4026700 là của ai?
-Vui lòng Những thông tin chi tiết của customer_account có mã số khách hàng với tài khoản là 6933679
-Vui lòng Lọc các thông tin chi tiết của customer_account có customer_no là 7281784
-Người dùng muốn tra cứu danh sách các giao dịch mua sắm theo số tài khoản nguồn.
-Các mã số khách hàng với tài khoản 6933679 là của ai?</t>
-  </si>
-  <si>
-    <t>Lọc customer_account có ngày hết hạn của tài khoản hoặc ngày đóng tài khoản trong khoảng 2026-01-28 - 2026-02-06
-Lọc customer_account có end_date trong khoảng 2026-01-29 - 2026-02-06
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-26 tới 2026-02-06
-Người dùng muốn tra cứu các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
-Người dùng muốn tra cứu danh sách các giao dịch nạp hoặc rút tiền theo số tài khoản nhận tiền hoặc tài khoản đích.
-Sao kê customer_account theo ngày end từ ngày 2025-12-22 đến ngày 2026-02-06
-Lọc customer_account có ngày nội dung trong khoảng 2026-01-26 - 2026-02-06
-Xem lịch sử customer_account dựa trên ngày end từ 2025-12-22 tới 2026-02-06
-Sao kê customer_account theo end_date từ ngày 2026-01-29 đến ngày 2026-02-06
-Xem lịch sử customer_account dựa trên ngày nội dung từ 2026-01-17 tới 2026-02-06</t>
-  </si>
-  <si>
-    <t>khách hàng bên lõi, số nội dung khách hàng, core_customer_id, mã nội dung khách hàng, id của khách hàng bên hệ thống lõi, core banking, mã core khách hàng, id khách hàng bên lõi map tài khoản với khách hàng</t>
-  </si>
-  <si>
-    <t>account_no, số tài khoản hoặc số thẻ, số tài khoản, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, số tài khoản số thẻ</t>
-  </si>
-  <si>
-    <t>tài khoản tiết kiệm, phân loại tài khoản, account_class, tài khoản thanh toán, thẻ tín dụng..., loại tài khoản</t>
-  </si>
-  <si>
-    <t>số order, order_no, số thứ tự hiển thị tài khoản trên giao diện, số trạng thái, số thứ tự hiển thị của tài khoản trên giao diện, app/web</t>
-  </si>
-  <si>
-    <t>a - active, trạng thái tài khoản, trạng thái, trạng thái bản ghi, status, i - inactive, c - closed</t>
-  </si>
-  <si>
-    <t>đã xác minh thông tin hay chưa, trạng thái verify, verify_status, trạng thái xác thực tài khoản, trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>trạng thái check, check_status, trạng thái kiểm tra, mặc định là 'u' - unknown hoặc unchecked, trạng thái trạng thái</t>
-  </si>
-  <si>
-    <t>ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày nội dung, create_date, ngày create, ngày mở tài khoản hoặc ngày bản ghi tạo</t>
-  </si>
-  <si>
-    <t>account_name, thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản</t>
+Xem lịch sử customer_account dựa trên ngày end từ 2026-01-14 tới 2026-02-09
+Sao kê customer_account theo ngày nội dung từ ngày 2026-02-08 đến ngày 2026-02-09
+Lọc customer_account có ngày nội dung trong khoảng 2026-02-08 - 2026-02-09
+Xem lịch sử customer_account dựa trên ngày end từ 2026-01-30 tới 2026-02-09
+Sao kê customer_account theo end_date từ ngày 2026-01-01 đến ngày 2026-02-09
+Xem lịch sử customer_account dựa trên ngày end từ 2025-12-11 tới 2026-02-09
+Người dùng muốn tra cứu một giao dịch nạp hoặc rút tiền cụ thể dựa trên mã nguồn hoặc mã tham chiếu.</t>
+  </si>
+  <si>
+    <t>core_customer_id, số nội dung khách hàng, core banking, id của khách hàng bên hệ thống lõi, mã core khách hàng, mã nội dung khách hàng, khách hàng bên lõi, id khách hàng bên lõi map tài khoản với khách hàng</t>
+  </si>
+  <si>
+    <t>số tài khoản số thẻ, số tài khoản, số tài khoản hoặc số thẻ đây là định danh tài khoản để giao dịch, account_no, số tài khoản hoặc số thẻ</t>
+  </si>
+  <si>
+    <t>tài khoản tiết kiệm, loại tài khoản, account_class, thẻ tín dụng..., phân loại tài khoản, tài khoản thanh toán</t>
+  </si>
+  <si>
+    <t>app/web, số order, order_no, số thứ tự hiển thị tài khoản trên giao diện, số trạng thái, số thứ tự hiển thị của tài khoản trên giao diện</t>
+  </si>
+  <si>
+    <t>c - closed, trạng thái, trạng thái tài khoản, trạng thái bản ghi, status, i - inactive, a - active</t>
+  </si>
+  <si>
+    <t>trạng thái verify, trạng thái trạng thái, verify_status, trạng thái xác thực tài khoản, đã xác minh thông tin hay chưa</t>
+  </si>
+  <si>
+    <t>trạng thái kiểm tra, trạng thái check, trạng thái trạng thái, check_status, mặc định là 'u' - unknown hoặc unchecked</t>
+  </si>
+  <si>
+    <t>create_date, ngày mở tài khoản hoặc ngày bản ghi được tạo, ngày create, ngày mở tài khoản hoặc ngày bản ghi tạo, ngày nội dung</t>
+  </si>
+  <si>
+    <t>thường là tên chủ tài khoản hoặc tên gợi nhớ, tên tài khoản, account_name</t>
   </si>
   <si>
     <t>tài khoản chi nhánh, account_branch, mã chi nhánh nơi quản lý tài khoản này</t>
   </si>
   <si>
-    <t>card_mask, số thẻ che bớt để đảm bảo bảo mật, số thẻ được che bớt, số tài khoản mask, card mask, 411122****1234</t>
-  </si>
-  <si>
-    <t>customer number, số khách hàng, customer_no, mã số khách hàng, mã số khách hàng với tài khoản</t>
-  </si>
-  <si>
-    <t>end_date, ngày end, ngày nội dung, ngày hết hạn tài khoản hoặc ngày đóng tài khoản, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản</t>
+    <t>411122****1234, số thẻ được che bớt, số tài khoản mask, card_mask, số thẻ che bớt để đảm bảo bảo mật, card mask</t>
+  </si>
+  <si>
+    <t>mã số khách hàng với tài khoản, số khách hàng, mã số khách hàng, customer number, customer_no</t>
+  </si>
+  <si>
+    <t>ngày end, ngày hết hạn của tài khoản hoặc ngày đóng tài khoản, end_date, ngày hết hạn tài khoản hoặc ngày đóng tài khoản, ngày nội dung</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer_account WHERE core_customer_id = '{{core_customer_id}}'"}</t>

</xml_diff>